<commit_message>
feat: make ARIA an installable PWA (icons + manifest)
- Generate square branded app icons (192/512/apple-touch) from the ARIA mark
- Update manifest: ARIA name, orange theme, any+maskable icon purposes
- Add mobile-web-app-capable meta; apple-touch-icon points to 180px asset
- Advisors can now 'Add to Home Screen' on Android & iPhone for an app-like
  full-screen experience

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/3_Portfolio_Holdings.xlsx
+++ b/notion-import-templates/3_Portfolio_Holdings.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24584D6D-82EB-4678-AC0C-52B4216DDD2A}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0F5BCCA-DFB4-4CC6-8817-A5B3F1BAA7BC}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="95">
   <si>
     <t/>
   </si>
@@ -310,6 +310,12 @@
   <si>
     <t>1. Manulife India Equity Fund - RM
 2. Phillip Master Money Market Fund</t>
+  </si>
+  <si>
+    <t>DORIS CHIEW JING TZE</t>
+  </si>
+  <si>
+    <t>Manulife Investment Greater China Fund</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -2917,14 +2923,30 @@
       </c>
     </row>
     <row r="39" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5"/>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-      <c r="E39" s="5"/>
-      <c r="F39" s="5"/>
-      <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
+      <c r="A39" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G39" s="21">
+        <v>12152.55</v>
+      </c>
+      <c r="H39" s="21">
+        <v>9000</v>
+      </c>
       <c r="I39" s="5"/>
       <c r="J39" s="14">
         <f t="shared" si="6"/>
@@ -2945,14 +2967,30 @@
       </c>
     </row>
     <row r="40" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
+      <c r="A40" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G40" s="21">
+        <v>3766.64</v>
+      </c>
+      <c r="H40" s="21">
+        <v>2000</v>
+      </c>
       <c r="I40" s="5"/>
       <c r="J40" s="14">
         <f t="shared" si="6"/>
@@ -3366,7 +3404,7 @@
     </row>
     <row r="55" spans="1:14" ht="26.1" customHeight="1">
       <c r="A55" s="18" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B55" s="18" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
feat: in-app Install ARIA prompt (Android native + iOS hint)
Mobile-only, dismissible banner: triggers the native install on Android/Chrome
via beforeinstallprompt; shows Add-to-Home-Screen hint on iOS Safari. Hidden
when already installed (standalone) or recently dismissed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/3_Portfolio_Holdings.xlsx
+++ b/notion-import-templates/3_Portfolio_Holdings.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0F5BCCA-DFB4-4CC6-8817-A5B3F1BAA7BC}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB7776D8-0CA3-4DC3-8524-E5F8B05F8B84}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="95">
   <si>
     <t/>
   </si>
@@ -3012,12 +3012,24 @@
     </row>
     <row r="41" spans="1:14" ht="22.15" customHeight="1">
       <c r="A41" s="5"/>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
+      <c r="B41" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G41" s="5">
+        <v>4.83</v>
+      </c>
       <c r="H41" s="5"/>
       <c r="I41" s="5"/>
       <c r="J41" s="14">

</xml_diff>

<commit_message>
feat: confirm tasks before adding via Ask ARIA
Ask ARIA now proposes extracted tasks for review instead of auto-creating
them. The advisor sees an editable card (task text, client, due date) — the
client field is highlighted when blank — and clicks Add to commit. Dashboard
task widget refreshes after adding.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/3_Portfolio_Holdings.xlsx
+++ b/notion-import-templates/3_Portfolio_Holdings.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB7776D8-0CA3-4DC3-8524-E5F8B05F8B84}"/>
+  <xr:revisionPtr revIDLastSave="86" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1063C796-8D07-44F8-AD3B-1CF7AEC93C70}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="97">
   <si>
     <t/>
   </si>
@@ -316,6 +316,12 @@
   </si>
   <si>
     <t>Manulife Investment Greater China Fund</t>
+  </si>
+  <si>
+    <t>TAN PIEH FANG</t>
+  </si>
+  <si>
+    <t>Cash Account</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -3011,7 +3017,9 @@
       </c>
     </row>
     <row r="41" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A41" s="5"/>
+      <c r="A41" s="5" t="s">
+        <v>92</v>
+      </c>
       <c r="B41" s="5" t="s">
         <v>80</v>
       </c>
@@ -3030,7 +3038,9 @@
       <c r="G41" s="5">
         <v>4.83</v>
       </c>
-      <c r="H41" s="5"/>
+      <c r="H41" s="5">
+        <v>61000</v>
+      </c>
       <c r="I41" s="5"/>
       <c r="J41" s="14">
         <f t="shared" si="6"/>
@@ -3051,14 +3061,30 @@
       </c>
     </row>
     <row r="42" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A42" s="5"/>
-      <c r="B42" s="5"/>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
+      <c r="A42" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G42" s="21">
+        <v>38798.160000000003</v>
+      </c>
+      <c r="H42" s="21">
+        <v>36000</v>
+      </c>
       <c r="I42" s="5"/>
       <c r="J42" s="14">
         <f t="shared" si="6"/>
@@ -3079,14 +3105,30 @@
       </c>
     </row>
     <row r="43" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A43" s="5"/>
-      <c r="B43" s="5"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="5"/>
-      <c r="G43" s="5"/>
-      <c r="H43" s="5"/>
+      <c r="A43" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F43" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G43" s="21">
+        <v>98857.14</v>
+      </c>
+      <c r="H43" s="21">
+        <v>94600</v>
+      </c>
       <c r="I43" s="5"/>
       <c r="J43" s="14">
         <f t="shared" si="6"/>
@@ -3107,14 +3149,30 @@
       </c>
     </row>
     <row r="44" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-      <c r="E44" s="5"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
+      <c r="A44" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G44" s="5">
+        <v>3.83</v>
+      </c>
+      <c r="H44" s="5">
+        <v>3.83</v>
+      </c>
       <c r="I44" s="5"/>
       <c r="J44" s="14">
         <f t="shared" si="6"/>
@@ -3135,14 +3193,30 @@
       </c>
     </row>
     <row r="45" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A45" s="5"/>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
-      <c r="E45" s="5"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
+      <c r="A45" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G45" s="5">
+        <v>8.56</v>
+      </c>
+      <c r="H45" s="5">
+        <v>8.56</v>
+      </c>
       <c r="I45" s="5"/>
       <c r="J45" s="14">
         <f t="shared" si="6"/>
@@ -3416,7 +3490,7 @@
     </row>
     <row r="55" spans="1:14" ht="26.1" customHeight="1">
       <c r="A55" s="18" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B55" s="18" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
ux: dashboard task completion shows checked + 'Done' before leaving list
Clicking the checkbox now briefly shows a green check, strikethrough and
'✓ Done' (0.9s) so it's clear the task was completed (moved to Done), not
deleted, before it slides off the open list.
</commit_message>
<xml_diff>
--- a/notion-import-templates/3_Portfolio_Holdings.xlsx
+++ b/notion-import-templates/3_Portfolio_Holdings.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="86" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1063C796-8D07-44F8-AD3B-1CF7AEC93C70}"/>
+  <xr:revisionPtr revIDLastSave="104" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{403B4EF1-E938-4F30-9F97-D76684F8BDF9}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="99">
   <si>
     <t/>
   </si>
@@ -322,6 +322,12 @@
   </si>
   <si>
     <t>Cash Account</t>
+  </si>
+  <si>
+    <t>Eastspring Investments Dinasti Equity Fund</t>
+  </si>
+  <si>
+    <t>Eastspring Investments Small-Cap Fund</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -3237,14 +3243,30 @@
       </c>
     </row>
     <row r="46" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A46" s="5"/>
-      <c r="B46" s="5"/>
-      <c r="C46" s="5"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="5"/>
-      <c r="H46" s="5"/>
+      <c r="A46" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G46" s="5">
+        <v>3.83</v>
+      </c>
+      <c r="H46" s="5">
+        <v>3.83</v>
+      </c>
       <c r="I46" s="5"/>
       <c r="J46" s="14">
         <f t="shared" si="6"/>
@@ -3265,14 +3287,30 @@
       </c>
     </row>
     <row r="47" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A47" s="5"/>
-      <c r="B47" s="5"/>
-      <c r="C47" s="5"/>
-      <c r="D47" s="5"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="5"/>
-      <c r="H47" s="5"/>
+      <c r="A47" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G47" s="5">
+        <v>3.83</v>
+      </c>
+      <c r="H47" s="5">
+        <v>3.83</v>
+      </c>
       <c r="I47" s="5"/>
       <c r="J47" s="14">
         <f t="shared" si="6"/>
@@ -3293,14 +3331,30 @@
       </c>
     </row>
     <row r="48" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5"/>
+      <c r="A48" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G48" s="21">
+        <v>66699.27</v>
+      </c>
+      <c r="H48" s="21">
+        <v>53168.06</v>
+      </c>
       <c r="I48" s="5"/>
       <c r="J48" s="14">
         <f t="shared" si="6"/>
@@ -3321,14 +3375,30 @@
       </c>
     </row>
     <row r="49" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A49" s="5"/>
-      <c r="B49" s="5"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
+      <c r="A49" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G49" s="21">
+        <v>32214.85</v>
+      </c>
+      <c r="H49" s="21">
+        <v>25901.95</v>
+      </c>
       <c r="I49" s="5"/>
       <c r="J49" s="14">
         <f t="shared" si="6"/>
@@ -3490,7 +3560,7 @@
     </row>
     <row r="55" spans="1:14" ht="26.1" customHeight="1">
       <c r="A55" s="18" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B55" s="18" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
ux: smaller, non-wrapping topbar date + Live Data badge on mobile/PWA
Date badge was 15px and could crowd/wrap on phones. Now 12px with no-wrap,
and the Live Data badge shrinks too, on screens <=768px.
</commit_message>
<xml_diff>
--- a/notion-import-templates/3_Portfolio_Holdings.xlsx
+++ b/notion-import-templates/3_Portfolio_Holdings.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30126"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="104" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{403B4EF1-E938-4F30-9F97-D76684F8BDF9}"/>
+  <xr:revisionPtr revIDLastSave="115" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA4D3274-F9F2-4AB4-B380-3EE119B2623F}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="101">
   <si>
     <t/>
   </si>
@@ -328,6 +328,12 @@
   </si>
   <si>
     <t>Eastspring Investments Small-Cap Fund</t>
+  </si>
+  <si>
+    <t>CBAAU 6.400% 05Mar2046 Corp (AUD)</t>
+  </si>
+  <si>
+    <t>AHAM AIIMAN PRS Shariah Growth Fund (PRS)</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -3419,14 +3425,30 @@
       </c>
     </row>
     <row r="50" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A50" s="5"/>
-      <c r="B50" s="5"/>
-      <c r="C50" s="5"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
-      <c r="G50" s="5"/>
-      <c r="H50" s="5"/>
+      <c r="A50" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="G50" s="21">
+        <v>19897</v>
+      </c>
+      <c r="H50" s="22">
+        <v>20000</v>
+      </c>
       <c r="I50" s="5"/>
       <c r="J50" s="14">
         <f t="shared" si="6"/>
@@ -3447,9 +3469,15 @@
       </c>
     </row>
     <row r="51" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A51" s="5"/>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
+      <c r="A51" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>66</v>
+      </c>
       <c r="D51" s="5"/>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
@@ -3560,7 +3588,7 @@
     </row>
     <row r="55" spans="1:14" ht="26.1" customHeight="1">
       <c r="A55" s="18" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B55" s="18" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
ux: Investment page — drop redundant per-row client column
The client name already appears in each group's header row (with avatar), so
the truncated per-row Client column was redundant. Removed it from the header,
rows, subtotal and grand total — giving holdings more room to display.
</commit_message>
<xml_diff>
--- a/notion-import-templates/3_Portfolio_Holdings.xlsx
+++ b/notion-import-templates/3_Portfolio_Holdings.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="382" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4A03FBC-5849-427D-9E9F-38EB3237FC1C}"/>
+  <xr:revisionPtr revIDLastSave="385" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91AC5B45-519D-430C-A88A-1D180417C7FD}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -392,7 +392,7 @@
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -610,7 +610,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -669,29 +669,28 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1033,14 +1032,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C29"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" ht="20.65">
+    <row r="2" spans="1:3" ht="20.65" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1051,7 +1050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1062,7 +1061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -1073,7 +1072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -1084,7 +1083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -1095,7 +1094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -1106,7 +1105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="25.5">
+    <row r="9" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -1117,7 +1116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="25.5">
+    <row r="10" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -1128,7 +1127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="25.5">
+    <row r="11" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1139,7 +1138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1150,7 +1149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -1161,7 +1160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="25.5">
+    <row r="14" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -1172,7 +1171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1183,7 +1182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -1194,7 +1193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -1205,7 +1204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1216,7 +1215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>0</v>
       </c>
@@ -1227,7 +1226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -1238,7 +1237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -1249,7 +1248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1260,7 +1259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="25.5">
+    <row r="25" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -1271,7 +1270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="25.5">
+    <row r="26" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -1282,7 +1281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="25.5">
+    <row r="27" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -1293,7 +1292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="25.5">
+    <row r="28" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>0</v>
       </c>
@@ -1304,7 +1303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="25.5">
+    <row r="29" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>0</v>
       </c>
@@ -1323,11 +1322,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N90"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:N89"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="54.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="54.265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="29" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
@@ -1341,43 +1340,43 @@
     <col min="14" max="14" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.15" customHeight="1">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:14" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-    </row>
-    <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1">
-      <c r="A2" s="25" t="s">
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+    </row>
+    <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
-    </row>
-    <row r="3" spans="1:14" ht="32.1" customHeight="1">
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+    </row>
+    <row r="3" spans="1:14" ht="32.1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="10" t="s">
         <v>28</v>
       </c>
@@ -1421,7 +1420,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="28.15" customHeight="1">
+    <row r="4" spans="1:14" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="13" t="s">
         <v>42</v>
       </c>
@@ -1465,7 +1464,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="22.15" customHeight="1">
+    <row r="5" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="5" t="s">
         <v>55</v>
       </c>
@@ -1511,7 +1510,7 @@
         <v>0.81413355794360354</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="22.15" customHeight="1">
+    <row r="6" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="5" t="s">
         <v>61</v>
       </c>
@@ -1547,7 +1546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="22.15" customHeight="1">
+    <row r="7" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="5" t="s">
         <v>63</v>
       </c>
@@ -1583,7 +1582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="22.15" customHeight="1">
+    <row r="8" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="5" t="s">
         <v>64</v>
       </c>
@@ -1629,7 +1628,7 @@
         <v>0.31638285714285719</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="22.15" customHeight="1">
+    <row r="9" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
         <v>67</v>
       </c>
@@ -1675,7 +1674,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="22.15" customHeight="1">
+    <row r="10" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="5" t="s">
         <v>55</v>
       </c>
@@ -1721,7 +1720,7 @@
         <v>2.115999999999996E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="22.15" customHeight="1">
+    <row r="11" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
         <v>55</v>
       </c>
@@ -1767,7 +1766,7 @@
         <v>0.70171076923076936</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="22.15" customHeight="1">
+    <row r="12" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="5" t="s">
         <v>55</v>
       </c>
@@ -1813,7 +1812,7 @@
         <v>8.044813559322038E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="22.15" customHeight="1">
+    <row r="13" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -1859,7 +1858,7 @@
         <v>7.6937391304347846E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="22.15" customHeight="1">
+    <row r="14" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
         <v>55</v>
       </c>
@@ -1905,7 +1904,7 @@
         <v>0.23820344424635223</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="22.15" customHeight="1">
+    <row r="15" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
         <v>55</v>
       </c>
@@ -1951,7 +1950,7 @@
         <v>-3.4960866666666701E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="22.15" customHeight="1">
+    <row r="16" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="5" t="s">
         <v>55</v>
       </c>
@@ -1997,7 +1996,7 @@
         <v>0.33413971962616829</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="22.15" customHeight="1">
+    <row r="17" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="5" t="s">
         <v>61</v>
       </c>
@@ -2043,7 +2042,7 @@
         <v>0.75419066666666668</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="22.15" customHeight="1">
+    <row r="18" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="5" t="s">
         <v>61</v>
       </c>
@@ -2089,7 +2088,7 @@
         <v>8.0448192771084337E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="22.15" customHeight="1">
+    <row r="19" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="5" t="s">
         <v>61</v>
       </c>
@@ -2135,7 +2134,7 @@
         <v>4.9483352468427097E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="22.15" customHeight="1">
+    <row r="20" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="5" t="s">
         <v>61</v>
       </c>
@@ -2181,7 +2180,7 @@
         <v>0.41930928987468363</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="22.15" customHeight="1">
+    <row r="21" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="5" t="s">
         <v>61</v>
       </c>
@@ -2227,7 +2226,7 @@
         <v>8.5334109223917844E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="22.15" customHeight="1">
+    <row r="22" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="5" t="s">
         <v>63</v>
       </c>
@@ -2273,7 +2272,7 @@
         <v>0.75419099999999994</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="22.15" customHeight="1">
+    <row r="23" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="5" t="s">
         <v>63</v>
       </c>
@@ -2319,7 +2318,7 @@
         <v>8.0448473282442742E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="22.15" customHeight="1">
+    <row r="24" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="5" t="s">
         <v>63</v>
       </c>
@@ -2365,7 +2364,7 @@
         <v>0.41841675268897716</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="22.15" customHeight="1">
+    <row r="25" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="5" t="s">
         <v>63</v>
       </c>
@@ -2411,7 +2410,7 @@
         <v>8.4817043627442735E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="22.15" customHeight="1">
+    <row r="26" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="5" t="s">
         <v>64</v>
       </c>
@@ -2457,7 +2456,7 @@
         <v>7.7633806146572185E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="22.15" customHeight="1">
+    <row r="27" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="5" t="s">
         <v>64</v>
       </c>
@@ -2503,7 +2502,7 @@
         <v>5.2741735537189423E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="22.15" customHeight="1">
+    <row r="28" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="5" t="s">
         <v>64</v>
       </c>
@@ -2549,7 +2548,7 @@
         <v>0.39329555555555556</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="22.15" customHeight="1">
+    <row r="29" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="5" t="s">
         <v>64</v>
       </c>
@@ -2589,7 +2588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="22.15" customHeight="1">
+    <row r="30" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="5" t="s">
         <v>67</v>
       </c>
@@ -2635,7 +2634,7 @@
         <v>0.15268291916376459</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="22.15" customHeight="1">
+    <row r="31" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="5" t="s">
         <v>67</v>
       </c>
@@ -2681,7 +2680,7 @@
         <v>0.29576248974094027</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="25.5">
+    <row r="32" spans="1:14" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A32" s="5" t="s">
         <v>83</v>
       </c>
@@ -2727,7 +2726,7 @@
         <v>-0.99778234042553182</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="22.15" customHeight="1">
+    <row r="33" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="5" t="s">
         <v>83</v>
       </c>
@@ -2773,7 +2772,7 @@
         <v>0.2698421508733983</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="22.15" customHeight="1">
+    <row r="34" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="5" t="s">
         <v>86</v>
       </c>
@@ -2819,7 +2818,7 @@
         <v>0.1016704587840358</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="22.15" customHeight="1">
+    <row r="35" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="5" t="s">
         <v>86</v>
       </c>
@@ -2865,7 +2864,7 @@
         <v>0.18256140350877198</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="22.15" customHeight="1">
+    <row r="36" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="5" t="s">
         <v>88</v>
       </c>
@@ -2911,7 +2910,7 @@
         <v>0.36689935589054251</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="22.15" customHeight="1">
+    <row r="37" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="5" t="s">
         <v>90</v>
       </c>
@@ -2940,11 +2939,11 @@
         <v>1</v>
       </c>
       <c r="J37" s="14">
-        <f t="shared" ref="J37:J54" si="6">G37*I37</f>
+        <f t="shared" ref="J37:J88" si="6">G37*I37</f>
         <v>6.9</v>
       </c>
       <c r="K37" s="14">
-        <f t="shared" ref="K37:K54" si="7">H37*I37</f>
+        <f t="shared" ref="K37:K88" si="7">H37*I37</f>
         <v>17000</v>
       </c>
       <c r="L37" s="15"/>
@@ -2957,7 +2956,7 @@
         <v>-0.99959411764705874</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="22.15" customHeight="1">
+    <row r="38" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="5" t="s">
         <v>90</v>
       </c>
@@ -3003,7 +3002,7 @@
         <v>-0.9997466647598422</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="22.15" customHeight="1">
+    <row r="39" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="5" t="s">
         <v>92</v>
       </c>
@@ -3028,26 +3027,28 @@
       <c r="H39" s="21">
         <v>9000</v>
       </c>
-      <c r="I39" s="5"/>
+      <c r="I39" s="5">
+        <v>1</v>
+      </c>
       <c r="J39" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>12152.55</v>
       </c>
       <c r="K39" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="L39" s="15"/>
       <c r="M39" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>3152.5499999999993</v>
       </c>
       <c r="N39" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="22.15" customHeight="1">
+        <v>0.35028333333333328</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="5" t="s">
         <v>92</v>
       </c>
@@ -3072,26 +3073,28 @@
       <c r="H40" s="21">
         <v>2000</v>
       </c>
-      <c r="I40" s="5"/>
+      <c r="I40" s="5">
+        <v>1</v>
+      </c>
       <c r="J40" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>3766.64</v>
       </c>
       <c r="K40" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="L40" s="15"/>
       <c r="M40" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1766.6399999999999</v>
       </c>
       <c r="N40" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" ht="22.15" customHeight="1">
+        <v>0.88331999999999988</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="5" t="s">
         <v>92</v>
       </c>
@@ -3116,26 +3119,28 @@
       <c r="H41" s="5">
         <v>61000</v>
       </c>
-      <c r="I41" s="5"/>
+      <c r="I41" s="5">
+        <v>1</v>
+      </c>
       <c r="J41" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>4.83</v>
       </c>
       <c r="K41" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>61000</v>
       </c>
       <c r="L41" s="15"/>
       <c r="M41" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>-60995.17</v>
       </c>
       <c r="N41" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" ht="22.15" customHeight="1">
+        <v>-0.99992081967213109</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="5" t="s">
         <v>94</v>
       </c>
@@ -3160,26 +3165,28 @@
       <c r="H42" s="21">
         <v>36000</v>
       </c>
-      <c r="I42" s="5"/>
+      <c r="I42" s="5">
+        <v>1</v>
+      </c>
       <c r="J42" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>38798.160000000003</v>
       </c>
       <c r="K42" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>36000</v>
       </c>
       <c r="L42" s="15"/>
       <c r="M42" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2798.1600000000035</v>
       </c>
       <c r="N42" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" ht="22.15" customHeight="1">
+        <v>7.7726666666666763E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="5" t="s">
         <v>94</v>
       </c>
@@ -3204,26 +3211,28 @@
       <c r="H43" s="21">
         <v>94600</v>
       </c>
-      <c r="I43" s="5"/>
+      <c r="I43" s="5">
+        <v>1</v>
+      </c>
       <c r="J43" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>98857.14</v>
       </c>
       <c r="K43" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>94600</v>
       </c>
       <c r="L43" s="15"/>
       <c r="M43" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>4257.1399999999994</v>
       </c>
       <c r="N43" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" ht="22.15" customHeight="1">
+        <v>4.50014799154334E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="5" t="s">
         <v>94</v>
       </c>
@@ -3248,14 +3257,16 @@
       <c r="H44" s="5">
         <v>3.83</v>
       </c>
-      <c r="I44" s="5"/>
+      <c r="I44" s="5">
+        <v>1</v>
+      </c>
       <c r="J44" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>3.83</v>
       </c>
       <c r="K44" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>3.83</v>
       </c>
       <c r="L44" s="15"/>
       <c r="M44" s="16">
@@ -3267,7 +3278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="22.15" customHeight="1">
+    <row r="45" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="5" t="s">
         <v>94</v>
       </c>
@@ -3292,14 +3303,16 @@
       <c r="H45" s="5">
         <v>8.56</v>
       </c>
-      <c r="I45" s="5"/>
+      <c r="I45" s="5">
+        <v>1</v>
+      </c>
       <c r="J45" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>8.56</v>
       </c>
       <c r="K45" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>8.56</v>
       </c>
       <c r="L45" s="15"/>
       <c r="M45" s="16">
@@ -3311,7 +3324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="22.15" customHeight="1">
+    <row r="46" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="5" t="s">
         <v>94</v>
       </c>
@@ -3336,14 +3349,16 @@
       <c r="H46" s="5">
         <v>3.83</v>
       </c>
-      <c r="I46" s="5"/>
+      <c r="I46" s="5">
+        <v>1</v>
+      </c>
       <c r="J46" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>3.83</v>
       </c>
       <c r="K46" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>3.83</v>
       </c>
       <c r="L46" s="15"/>
       <c r="M46" s="16">
@@ -3355,7 +3370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="22.15" customHeight="1">
+    <row r="47" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="5" t="s">
         <v>94</v>
       </c>
@@ -3380,14 +3395,16 @@
       <c r="H47" s="5">
         <v>3.83</v>
       </c>
-      <c r="I47" s="5"/>
+      <c r="I47" s="5">
+        <v>1</v>
+      </c>
       <c r="J47" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>3.83</v>
       </c>
       <c r="K47" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>3.83</v>
       </c>
       <c r="L47" s="15"/>
       <c r="M47" s="16">
@@ -3399,7 +3416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="22.15" customHeight="1">
+    <row r="48" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="5" t="s">
         <v>94</v>
       </c>
@@ -3424,26 +3441,28 @@
       <c r="H48" s="21">
         <v>53168.06</v>
       </c>
-      <c r="I48" s="5"/>
+      <c r="I48" s="5">
+        <v>1</v>
+      </c>
       <c r="J48" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>66699.27</v>
       </c>
       <c r="K48" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>53168.06</v>
       </c>
       <c r="L48" s="15"/>
       <c r="M48" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>13531.210000000006</v>
       </c>
       <c r="N48" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:14" ht="22.15" customHeight="1">
+        <v>0.25449884761640745</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="5" t="s">
         <v>94</v>
       </c>
@@ -3468,26 +3487,28 @@
       <c r="H49" s="21">
         <v>25901.95</v>
       </c>
-      <c r="I49" s="5"/>
+      <c r="I49" s="5">
+        <v>1</v>
+      </c>
       <c r="J49" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>32214.85</v>
       </c>
       <c r="K49" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>25901.95</v>
       </c>
       <c r="L49" s="15"/>
       <c r="M49" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>6312.8999999999978</v>
       </c>
       <c r="N49" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" ht="22.15" customHeight="1">
+        <v>0.24372296294294435</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="5" t="s">
         <v>94</v>
       </c>
@@ -3512,26 +3533,28 @@
       <c r="H50" s="22">
         <v>20000</v>
       </c>
-      <c r="I50" s="5"/>
+      <c r="I50" s="5">
+        <v>1</v>
+      </c>
       <c r="J50" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>19897</v>
       </c>
       <c r="K50" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="L50" s="15"/>
       <c r="M50" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>-103</v>
       </c>
       <c r="N50" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14" ht="22.15" customHeight="1">
+        <v>-5.1500000000000001E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="5" t="s">
         <v>94</v>
       </c>
@@ -3556,26 +3579,28 @@
       <c r="H51" s="21">
         <v>11177.8</v>
       </c>
-      <c r="I51" s="5"/>
+      <c r="I51" s="5">
+        <v>1</v>
+      </c>
       <c r="J51" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>15916.18</v>
       </c>
       <c r="K51" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>11177.8</v>
       </c>
       <c r="L51" s="15"/>
       <c r="M51" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>4738.380000000001</v>
       </c>
       <c r="N51" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" ht="22.15" customHeight="1">
+        <v>0.42390989282327485</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="5" t="s">
         <v>94</v>
       </c>
@@ -3600,26 +3625,28 @@
       <c r="H52" s="21">
         <v>17500</v>
       </c>
-      <c r="I52" s="5"/>
+      <c r="I52" s="5">
+        <v>1</v>
+      </c>
       <c r="J52" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>23276.19</v>
       </c>
       <c r="K52" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>17500</v>
       </c>
       <c r="L52" s="15"/>
       <c r="M52" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>5776.1899999999987</v>
       </c>
       <c r="N52" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:14" ht="22.15" customHeight="1">
+        <v>0.33006799999999992</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="5" t="s">
         <v>101</v>
       </c>
@@ -3644,26 +3671,28 @@
       <c r="H53" s="21">
         <v>25800</v>
       </c>
-      <c r="I53" s="5"/>
+      <c r="I53" s="5">
+        <v>1</v>
+      </c>
       <c r="J53" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>44041.25</v>
       </c>
       <c r="K53" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>25800</v>
       </c>
       <c r="L53" s="15"/>
       <c r="M53" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>18241.25</v>
       </c>
       <c r="N53" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:14" ht="22.15" customHeight="1">
+        <v>0.70702519379844964</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="5" t="s">
         <v>101</v>
       </c>
@@ -3688,30 +3717,32 @@
       <c r="H54" s="21">
         <v>55000</v>
       </c>
-      <c r="I54" s="5"/>
+      <c r="I54" s="5">
+        <v>1</v>
+      </c>
       <c r="J54" s="14">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>61289.25</v>
       </c>
       <c r="K54" s="14">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>55000</v>
       </c>
       <c r="L54" s="15"/>
       <c r="M54" s="16">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>6289.25</v>
       </c>
       <c r="N54" s="17">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" ht="22.15" customHeight="1">
+        <v>0.11434999999999999</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B55" s="26" t="s">
+      <c r="B55" s="24" t="s">
         <v>75</v>
       </c>
       <c r="C55" s="5" t="s">
@@ -3726,27 +3757,35 @@
       <c r="F55" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G55" s="31">
+      <c r="G55" s="28">
         <v>102950.64</v>
       </c>
-      <c r="H55" s="31">
+      <c r="H55" s="28">
         <v>94300</v>
       </c>
-      <c r="I55" s="26"/>
-      <c r="J55" s="27"/>
-      <c r="K55" s="27"/>
-      <c r="L55" s="28"/>
-      <c r="M55" s="29"/>
-      <c r="N55" s="30"/>
-    </row>
-    <row r="56" spans="1:14" ht="22.15" customHeight="1">
+      <c r="I55" s="5">
+        <v>1</v>
+      </c>
+      <c r="J55" s="14">
+        <f t="shared" si="6"/>
+        <v>102950.64</v>
+      </c>
+      <c r="K55" s="14">
+        <f t="shared" si="7"/>
+        <v>94300</v>
+      </c>
+      <c r="L55" s="25"/>
+      <c r="M55" s="26"/>
+      <c r="N55" s="27"/>
+    </row>
+    <row r="56" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B56" s="26" t="s">
+      <c r="B56" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C56" s="26" t="s">
+      <c r="C56" s="24" t="s">
         <v>57</v>
       </c>
       <c r="D56" s="5" t="s">
@@ -3758,27 +3797,35 @@
       <c r="F56" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G56" s="31">
+      <c r="G56" s="28">
         <v>160999.82</v>
       </c>
-      <c r="H56" s="31">
+      <c r="H56" s="28">
         <v>137600</v>
       </c>
-      <c r="I56" s="26"/>
-      <c r="J56" s="27"/>
-      <c r="K56" s="27"/>
-      <c r="L56" s="28"/>
-      <c r="M56" s="29"/>
-      <c r="N56" s="30"/>
-    </row>
-    <row r="57" spans="1:14" ht="22.15" customHeight="1">
+      <c r="I56" s="5">
+        <v>1</v>
+      </c>
+      <c r="J56" s="14">
+        <f t="shared" si="6"/>
+        <v>160999.82</v>
+      </c>
+      <c r="K56" s="14">
+        <f t="shared" si="7"/>
+        <v>137600</v>
+      </c>
+      <c r="L56" s="25"/>
+      <c r="M56" s="26"/>
+      <c r="N56" s="27"/>
+    </row>
+    <row r="57" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B57" s="26" t="s">
+      <c r="B57" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="C57" s="26" t="s">
+      <c r="C57" s="24" t="s">
         <v>57</v>
       </c>
       <c r="D57" s="5" t="s">
@@ -3790,91 +3837,115 @@
       <c r="F57" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G57" s="31">
+      <c r="G57" s="28">
         <v>10616.87</v>
       </c>
-      <c r="H57" s="31">
+      <c r="H57" s="28">
         <v>12100</v>
       </c>
-      <c r="I57" s="26"/>
-      <c r="J57" s="27"/>
-      <c r="K57" s="27"/>
-      <c r="L57" s="28"/>
-      <c r="M57" s="29"/>
-      <c r="N57" s="30"/>
-    </row>
-    <row r="58" spans="1:14" ht="22.15" customHeight="1">
+      <c r="I57" s="5">
+        <v>1</v>
+      </c>
+      <c r="J57" s="14">
+        <f t="shared" si="6"/>
+        <v>10616.87</v>
+      </c>
+      <c r="K57" s="14">
+        <f t="shared" si="7"/>
+        <v>12100</v>
+      </c>
+      <c r="L57" s="25"/>
+      <c r="M57" s="26"/>
+      <c r="N57" s="27"/>
+    </row>
+    <row r="58" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B58" s="26" t="s">
+      <c r="B58" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="C58" s="26" t="s">
+      <c r="C58" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D58" s="26" t="s">
+      <c r="D58" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E58" s="26" t="s">
+      <c r="E58" s="24" t="s">
         <v>59</v>
       </c>
       <c r="F58" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G58" s="31">
+      <c r="G58" s="28">
         <v>1296.3399999999999</v>
       </c>
-      <c r="H58" s="31">
+      <c r="H58" s="28">
         <v>1200</v>
       </c>
-      <c r="I58" s="26"/>
-      <c r="J58" s="27"/>
-      <c r="K58" s="27"/>
-      <c r="L58" s="28"/>
-      <c r="M58" s="29"/>
-      <c r="N58" s="30"/>
-    </row>
-    <row r="59" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A59" s="26" t="s">
+      <c r="I58" s="5">
+        <v>1</v>
+      </c>
+      <c r="J58" s="14">
+        <f t="shared" si="6"/>
+        <v>1296.3399999999999</v>
+      </c>
+      <c r="K58" s="14">
+        <f t="shared" si="7"/>
+        <v>1200</v>
+      </c>
+      <c r="L58" s="25"/>
+      <c r="M58" s="26"/>
+      <c r="N58" s="27"/>
+    </row>
+    <row r="59" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A59" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="B59" s="26" t="s">
+      <c r="B59" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="C59" s="26" t="s">
+      <c r="C59" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D59" s="26" t="s">
+      <c r="D59" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E59" s="26" t="s">
+      <c r="E59" s="24" t="s">
         <v>59</v>
       </c>
       <c r="F59" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G59" s="31">
+      <c r="G59" s="28">
         <v>4108.8500000000004</v>
       </c>
-      <c r="H59" s="31">
+      <c r="H59" s="28">
         <v>3000</v>
       </c>
-      <c r="I59" s="26"/>
-      <c r="J59" s="27"/>
-      <c r="K59" s="27"/>
-      <c r="L59" s="28"/>
-      <c r="M59" s="29"/>
-      <c r="N59" s="30"/>
-    </row>
-    <row r="60" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A60" s="26" t="s">
+      <c r="I59" s="5">
+        <v>1</v>
+      </c>
+      <c r="J59" s="14">
+        <f t="shared" si="6"/>
+        <v>4108.8500000000004</v>
+      </c>
+      <c r="K59" s="14">
+        <f t="shared" si="7"/>
+        <v>3000</v>
+      </c>
+      <c r="L59" s="25"/>
+      <c r="M59" s="26"/>
+      <c r="N59" s="27"/>
+    </row>
+    <row r="60" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A60" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="B60" s="26" t="s">
+      <c r="B60" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="C60" s="26" t="s">
+      <c r="C60" s="24" t="s">
         <v>57</v>
       </c>
       <c r="D60" s="5" t="s">
@@ -3886,27 +3957,35 @@
       <c r="F60" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G60" s="31">
+      <c r="G60" s="28">
         <v>16947.36</v>
       </c>
-      <c r="H60" s="31">
+      <c r="H60" s="28">
         <v>12800</v>
       </c>
-      <c r="I60" s="26"/>
-      <c r="J60" s="27"/>
-      <c r="K60" s="27"/>
-      <c r="L60" s="28"/>
-      <c r="M60" s="29"/>
-      <c r="N60" s="30"/>
-    </row>
-    <row r="61" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A61" s="26" t="s">
+      <c r="I60" s="5">
+        <v>1</v>
+      </c>
+      <c r="J60" s="14">
+        <f t="shared" si="6"/>
+        <v>16947.36</v>
+      </c>
+      <c r="K60" s="14">
+        <f t="shared" si="7"/>
+        <v>12800</v>
+      </c>
+      <c r="L60" s="25"/>
+      <c r="M60" s="26"/>
+      <c r="N60" s="27"/>
+    </row>
+    <row r="61" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A61" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="B61" s="26" t="s">
+      <c r="B61" s="24" t="s">
         <v>105</v>
       </c>
-      <c r="C61" s="26" t="s">
+      <c r="C61" s="24" t="s">
         <v>57</v>
       </c>
       <c r="D61" s="5" t="s">
@@ -3918,27 +3997,35 @@
       <c r="F61" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G61" s="31">
+      <c r="G61" s="28">
         <v>26937.05</v>
       </c>
-      <c r="H61" s="31">
+      <c r="H61" s="28">
         <v>17400</v>
       </c>
-      <c r="I61" s="26"/>
-      <c r="J61" s="27"/>
-      <c r="K61" s="27"/>
-      <c r="L61" s="28"/>
-      <c r="M61" s="29"/>
-      <c r="N61" s="30"/>
-    </row>
-    <row r="62" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A62" s="26" t="s">
+      <c r="I61" s="5">
+        <v>1</v>
+      </c>
+      <c r="J61" s="14">
+        <f t="shared" si="6"/>
+        <v>26937.05</v>
+      </c>
+      <c r="K61" s="14">
+        <f t="shared" si="7"/>
+        <v>17400</v>
+      </c>
+      <c r="L61" s="25"/>
+      <c r="M61" s="26"/>
+      <c r="N61" s="27"/>
+    </row>
+    <row r="62" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A62" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="B62" s="26" t="s">
+      <c r="B62" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="C62" s="26" t="s">
+      <c r="C62" s="24" t="s">
         <v>57</v>
       </c>
       <c r="D62" s="5" t="s">
@@ -3950,30 +4037,38 @@
       <c r="F62" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G62" s="31">
+      <c r="G62" s="28">
         <v>22790.720000000001</v>
       </c>
-      <c r="H62" s="32">
+      <c r="H62" s="29">
         <v>13700</v>
       </c>
-      <c r="I62" s="26"/>
-      <c r="J62" s="27"/>
-      <c r="K62" s="27"/>
-      <c r="L62" s="28"/>
-      <c r="M62" s="29"/>
-      <c r="N62" s="30"/>
-    </row>
-    <row r="63" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A63" s="26" t="s">
+      <c r="I62" s="5">
+        <v>1</v>
+      </c>
+      <c r="J62" s="14">
+        <f t="shared" si="6"/>
+        <v>22790.720000000001</v>
+      </c>
+      <c r="K62" s="14">
+        <f t="shared" si="7"/>
+        <v>13700</v>
+      </c>
+      <c r="L62" s="25"/>
+      <c r="M62" s="26"/>
+      <c r="N62" s="27"/>
+    </row>
+    <row r="63" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A63" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="B63" s="26" t="s">
+      <c r="B63" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C63" s="26" t="s">
+      <c r="C63" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D63" s="26" t="s">
+      <c r="D63" s="24" t="s">
         <v>78</v>
       </c>
       <c r="E63" s="5" t="s">
@@ -3982,27 +4077,35 @@
       <c r="F63" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G63" s="31">
+      <c r="G63" s="28">
         <v>51227.25</v>
       </c>
-      <c r="H63" s="31">
+      <c r="H63" s="28">
         <v>43000</v>
       </c>
-      <c r="I63" s="26"/>
-      <c r="J63" s="27"/>
-      <c r="K63" s="27"/>
-      <c r="L63" s="28"/>
-      <c r="M63" s="29"/>
-      <c r="N63" s="30"/>
-    </row>
-    <row r="64" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A64" s="26" t="s">
+      <c r="I63" s="5">
+        <v>1</v>
+      </c>
+      <c r="J63" s="14">
+        <f t="shared" si="6"/>
+        <v>51227.25</v>
+      </c>
+      <c r="K63" s="14">
+        <f t="shared" si="7"/>
+        <v>43000</v>
+      </c>
+      <c r="L63" s="25"/>
+      <c r="M63" s="26"/>
+      <c r="N63" s="27"/>
+    </row>
+    <row r="64" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A64" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="B64" s="26" t="s">
+      <c r="B64" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="C64" s="26" t="s">
+      <c r="C64" s="24" t="s">
         <v>57</v>
       </c>
       <c r="D64" s="5" t="s">
@@ -4014,30 +4117,38 @@
       <c r="F64" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G64" s="31">
+      <c r="G64" s="28">
         <v>26846.82</v>
       </c>
-      <c r="H64" s="31">
+      <c r="H64" s="28">
         <v>20600</v>
       </c>
-      <c r="I64" s="26"/>
-      <c r="J64" s="27"/>
-      <c r="K64" s="27"/>
-      <c r="L64" s="28"/>
-      <c r="M64" s="29"/>
-      <c r="N64" s="30"/>
-    </row>
-    <row r="65" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A65" s="26" t="s">
+      <c r="I64" s="5">
+        <v>1</v>
+      </c>
+      <c r="J64" s="14">
+        <f t="shared" si="6"/>
+        <v>26846.82</v>
+      </c>
+      <c r="K64" s="14">
+        <f t="shared" si="7"/>
+        <v>20600</v>
+      </c>
+      <c r="L64" s="25"/>
+      <c r="M64" s="26"/>
+      <c r="N64" s="27"/>
+    </row>
+    <row r="65" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A65" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="B65" s="26" t="s">
+      <c r="B65" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C65" s="26" t="s">
+      <c r="C65" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D65" s="26" t="s">
+      <c r="D65" s="24" t="s">
         <v>78</v>
       </c>
       <c r="E65" s="5" t="s">
@@ -4046,59 +4157,75 @@
       <c r="F65" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G65" s="31">
+      <c r="G65" s="28">
         <v>42050.239999999998</v>
       </c>
-      <c r="H65" s="31">
+      <c r="H65" s="28">
         <v>35900</v>
       </c>
-      <c r="I65" s="26"/>
-      <c r="J65" s="27"/>
-      <c r="K65" s="27"/>
-      <c r="L65" s="28"/>
-      <c r="M65" s="29"/>
-      <c r="N65" s="30"/>
-    </row>
-    <row r="66" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A66" s="26" t="s">
+      <c r="I65" s="5">
+        <v>1</v>
+      </c>
+      <c r="J65" s="14">
+        <f t="shared" si="6"/>
+        <v>42050.239999999998</v>
+      </c>
+      <c r="K65" s="14">
+        <f t="shared" si="7"/>
+        <v>35900</v>
+      </c>
+      <c r="L65" s="25"/>
+      <c r="M65" s="26"/>
+      <c r="N65" s="27"/>
+    </row>
+    <row r="66" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A66" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="B66" s="26" t="s">
+      <c r="B66" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="C66" s="26" t="s">
+      <c r="C66" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="D66" s="26" t="s">
+      <c r="D66" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E66" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F66" s="26" t="s">
+      <c r="E66" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F66" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="G66" s="31">
+      <c r="G66" s="28">
         <v>23922.5</v>
       </c>
-      <c r="H66" s="32">
+      <c r="H66" s="29">
         <v>25000</v>
       </c>
-      <c r="I66" s="26"/>
-      <c r="J66" s="27"/>
-      <c r="K66" s="27"/>
-      <c r="L66" s="28"/>
-      <c r="M66" s="29"/>
-      <c r="N66" s="30"/>
-    </row>
-    <row r="67" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A67" s="26" t="s">
+      <c r="I66" s="5">
+        <v>1</v>
+      </c>
+      <c r="J66" s="14">
+        <f t="shared" si="6"/>
+        <v>23922.5</v>
+      </c>
+      <c r="K66" s="14">
+        <f t="shared" si="7"/>
+        <v>25000</v>
+      </c>
+      <c r="L66" s="25"/>
+      <c r="M66" s="26"/>
+      <c r="N66" s="27"/>
+    </row>
+    <row r="67" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A67" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="B67" s="26" t="s">
+      <c r="B67" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="C67" s="26" t="s">
+      <c r="C67" s="24" t="s">
         <v>57</v>
       </c>
       <c r="D67" s="5" t="s">
@@ -4110,27 +4237,35 @@
       <c r="F67" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G67" s="31">
+      <c r="G67" s="28">
         <v>94261.19</v>
       </c>
-      <c r="H67" s="31">
+      <c r="H67" s="28">
         <v>90100</v>
       </c>
-      <c r="I67" s="26"/>
-      <c r="J67" s="27"/>
-      <c r="K67" s="27"/>
-      <c r="L67" s="28"/>
-      <c r="M67" s="29"/>
-      <c r="N67" s="30"/>
-    </row>
-    <row r="68" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A68" s="26" t="s">
+      <c r="I67" s="5">
+        <v>1</v>
+      </c>
+      <c r="J67" s="14">
+        <f t="shared" si="6"/>
+        <v>94261.19</v>
+      </c>
+      <c r="K67" s="14">
+        <f t="shared" si="7"/>
+        <v>90100</v>
+      </c>
+      <c r="L67" s="25"/>
+      <c r="M67" s="26"/>
+      <c r="N67" s="27"/>
+    </row>
+    <row r="68" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A68" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="B68" s="26" t="s">
+      <c r="B68" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="C68" s="26" t="s">
+      <c r="C68" s="24" t="s">
         <v>57</v>
       </c>
       <c r="D68" s="5" t="s">
@@ -4142,30 +4277,38 @@
       <c r="F68" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G68" s="31">
+      <c r="G68" s="28">
         <v>136256.26</v>
       </c>
-      <c r="H68" s="31">
+      <c r="H68" s="28">
         <v>128000</v>
       </c>
-      <c r="I68" s="26"/>
-      <c r="J68" s="27"/>
-      <c r="K68" s="27"/>
-      <c r="L68" s="28"/>
-      <c r="M68" s="29"/>
-      <c r="N68" s="30"/>
-    </row>
-    <row r="69" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A69" s="26" t="s">
+      <c r="I68" s="5">
+        <v>1</v>
+      </c>
+      <c r="J68" s="14">
+        <f t="shared" si="6"/>
+        <v>136256.26</v>
+      </c>
+      <c r="K68" s="14">
+        <f t="shared" si="7"/>
+        <v>128000</v>
+      </c>
+      <c r="L68" s="25"/>
+      <c r="M68" s="26"/>
+      <c r="N68" s="27"/>
+    </row>
+    <row r="69" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A69" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="B69" s="26" t="s">
+      <c r="B69" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C69" s="26" t="s">
+      <c r="C69" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D69" s="26" t="s">
+      <c r="D69" s="24" t="s">
         <v>58</v>
       </c>
       <c r="E69" s="5" t="s">
@@ -4174,27 +4317,35 @@
       <c r="F69" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G69" s="26">
+      <c r="G69" s="24">
         <v>4.32</v>
       </c>
-      <c r="H69" s="26">
+      <c r="H69" s="24">
         <v>4.32</v>
       </c>
-      <c r="I69" s="26"/>
-      <c r="J69" s="27"/>
-      <c r="K69" s="27"/>
-      <c r="L69" s="28"/>
-      <c r="M69" s="29"/>
-      <c r="N69" s="30"/>
-    </row>
-    <row r="70" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A70" s="26" t="s">
+      <c r="I69" s="5">
+        <v>1</v>
+      </c>
+      <c r="J69" s="14">
+        <f t="shared" si="6"/>
+        <v>4.32</v>
+      </c>
+      <c r="K69" s="14">
+        <f t="shared" si="7"/>
+        <v>4.32</v>
+      </c>
+      <c r="L69" s="25"/>
+      <c r="M69" s="26"/>
+      <c r="N69" s="27"/>
+    </row>
+    <row r="70" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A70" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="B70" s="26" t="s">
+      <c r="B70" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="C70" s="26" t="s">
+      <c r="C70" s="24" t="s">
         <v>66</v>
       </c>
       <c r="D70" s="5" t="s">
@@ -4206,27 +4357,35 @@
       <c r="F70" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G70" s="31">
+      <c r="G70" s="28">
         <v>3474.65</v>
       </c>
-      <c r="H70" s="26">
+      <c r="H70" s="24">
         <v>2500</v>
       </c>
-      <c r="I70" s="26"/>
-      <c r="J70" s="27"/>
-      <c r="K70" s="27"/>
-      <c r="L70" s="28"/>
-      <c r="M70" s="29"/>
-      <c r="N70" s="30"/>
-    </row>
-    <row r="71" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A71" s="26" t="s">
+      <c r="I70" s="5">
+        <v>1</v>
+      </c>
+      <c r="J70" s="14">
+        <f t="shared" si="6"/>
+        <v>3474.65</v>
+      </c>
+      <c r="K70" s="14">
+        <f t="shared" si="7"/>
+        <v>2500</v>
+      </c>
+      <c r="L70" s="25"/>
+      <c r="M70" s="26"/>
+      <c r="N70" s="27"/>
+    </row>
+    <row r="71" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A71" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="B71" s="26" t="s">
+      <c r="B71" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="C71" s="26" t="s">
+      <c r="C71" s="24" t="s">
         <v>66</v>
       </c>
       <c r="D71" s="5" t="s">
@@ -4238,560 +4397,704 @@
       <c r="F71" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G71" s="32">
+      <c r="G71" s="29">
         <v>34455</v>
       </c>
-      <c r="H71" s="31">
+      <c r="H71" s="28">
         <v>23935.360000000001</v>
       </c>
-      <c r="I71" s="26"/>
-      <c r="J71" s="27"/>
-      <c r="K71" s="27"/>
-      <c r="L71" s="28"/>
-      <c r="M71" s="29"/>
-      <c r="N71" s="30"/>
-    </row>
-    <row r="72" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A72" s="26" t="s">
+      <c r="I71" s="5">
+        <v>1</v>
+      </c>
+      <c r="J71" s="14">
+        <f t="shared" si="6"/>
+        <v>34455</v>
+      </c>
+      <c r="K71" s="14">
+        <f t="shared" si="7"/>
+        <v>23935.360000000001</v>
+      </c>
+      <c r="L71" s="25"/>
+      <c r="M71" s="26"/>
+      <c r="N71" s="27"/>
+    </row>
+    <row r="72" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A72" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="B72" s="26" t="s">
+      <c r="B72" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="C72" s="26" t="s">
+      <c r="C72" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="D72" s="26" t="s">
+      <c r="D72" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E72" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F72" s="26" t="s">
+      <c r="E72" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F72" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="G72" s="26">
+      <c r="G72" s="24">
         <v>25.6</v>
       </c>
-      <c r="H72" s="26">
+      <c r="H72" s="24">
         <v>20000</v>
       </c>
-      <c r="I72" s="26"/>
-      <c r="J72" s="27"/>
-      <c r="K72" s="27"/>
-      <c r="L72" s="28"/>
-      <c r="M72" s="29"/>
-      <c r="N72" s="30"/>
-    </row>
-    <row r="73" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A73" s="26" t="s">
+      <c r="I72" s="5">
+        <v>1</v>
+      </c>
+      <c r="J72" s="14">
+        <f t="shared" si="6"/>
+        <v>25.6</v>
+      </c>
+      <c r="K72" s="14">
+        <f t="shared" si="7"/>
+        <v>20000</v>
+      </c>
+      <c r="L72" s="25"/>
+      <c r="M72" s="26"/>
+      <c r="N72" s="27"/>
+    </row>
+    <row r="73" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A73" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="B73" s="26" t="s">
+      <c r="B73" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C73" s="26" t="s">
+      <c r="C73" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D73" s="26" t="s">
+      <c r="D73" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E73" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F73" s="26" t="s">
+      <c r="E73" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F73" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="G73" s="26">
+      <c r="G73" s="24">
         <v>34.49</v>
       </c>
-      <c r="H73" s="26">
+      <c r="H73" s="24">
         <v>34.49</v>
       </c>
-      <c r="I73" s="26"/>
-      <c r="J73" s="27"/>
-      <c r="K73" s="27"/>
-      <c r="L73" s="28"/>
-      <c r="M73" s="29"/>
-      <c r="N73" s="30"/>
-    </row>
-    <row r="74" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A74" s="26" t="s">
+      <c r="I73" s="5">
+        <v>1</v>
+      </c>
+      <c r="J73" s="14">
+        <f t="shared" si="6"/>
+        <v>34.49</v>
+      </c>
+      <c r="K73" s="14">
+        <f t="shared" si="7"/>
+        <v>34.49</v>
+      </c>
+      <c r="L73" s="25"/>
+      <c r="M73" s="26"/>
+      <c r="N73" s="27"/>
+    </row>
+    <row r="74" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A74" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="B74" s="26" t="s">
+      <c r="B74" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C74" s="26" t="s">
+      <c r="C74" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D74" s="26" t="s">
+      <c r="D74" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E74" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F74" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G74" s="26">
+      <c r="E74" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F74" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G74" s="24">
         <v>6.24</v>
       </c>
-      <c r="H74" s="26">
+      <c r="H74" s="24">
         <v>6.24</v>
       </c>
-      <c r="I74" s="26"/>
-      <c r="J74" s="27"/>
-      <c r="K74" s="27"/>
-      <c r="L74" s="28"/>
-      <c r="M74" s="29"/>
-      <c r="N74" s="30"/>
-    </row>
-    <row r="75" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A75" s="26" t="s">
+      <c r="I74" s="5">
+        <v>1</v>
+      </c>
+      <c r="J74" s="14">
+        <f t="shared" si="6"/>
+        <v>6.24</v>
+      </c>
+      <c r="K74" s="14">
+        <f t="shared" si="7"/>
+        <v>6.24</v>
+      </c>
+      <c r="L74" s="25"/>
+      <c r="M74" s="26"/>
+      <c r="N74" s="27"/>
+    </row>
+    <row r="75" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A75" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="B75" s="26" t="s">
+      <c r="B75" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C75" s="26" t="s">
+      <c r="C75" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D75" s="26" t="s">
+      <c r="D75" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="E75" s="26" t="s">
+      <c r="E75" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="F75" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G75" s="31"/>
-      <c r="H75" s="31"/>
-      <c r="I75" s="26"/>
-      <c r="J75" s="27"/>
-      <c r="K75" s="27"/>
-      <c r="L75" s="28"/>
-      <c r="M75" s="29"/>
-      <c r="N75" s="30"/>
-    </row>
-    <row r="76" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A76" s="26" t="s">
+      <c r="F75" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G75" s="28"/>
+      <c r="H75" s="28"/>
+      <c r="I75" s="5">
+        <v>1</v>
+      </c>
+      <c r="J75" s="14">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="K75" s="14">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="L75" s="25"/>
+      <c r="M75" s="26"/>
+      <c r="N75" s="27"/>
+    </row>
+    <row r="76" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A76" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="B76" s="26" t="s">
+      <c r="B76" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="C76" s="26" t="s">
+      <c r="C76" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D76" s="26" t="s">
+      <c r="D76" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E76" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F76" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G76" s="31">
+      <c r="E76" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F76" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G76" s="28">
         <v>17731.580000000002</v>
       </c>
-      <c r="H76" s="31">
+      <c r="H76" s="28">
         <v>14415.3</v>
       </c>
-      <c r="I76" s="26"/>
-      <c r="J76" s="27"/>
-      <c r="K76" s="27"/>
-      <c r="L76" s="28"/>
-      <c r="M76" s="29"/>
-      <c r="N76" s="30"/>
-    </row>
-    <row r="77" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A77" s="26" t="s">
+      <c r="I76" s="5">
+        <v>1</v>
+      </c>
+      <c r="J76" s="14">
+        <f t="shared" si="6"/>
+        <v>17731.580000000002</v>
+      </c>
+      <c r="K76" s="14">
+        <f t="shared" si="7"/>
+        <v>14415.3</v>
+      </c>
+      <c r="L76" s="25"/>
+      <c r="M76" s="26"/>
+      <c r="N76" s="27"/>
+    </row>
+    <row r="77" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A77" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="B77" s="26" t="s">
+      <c r="B77" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="C77" s="26" t="s">
+      <c r="C77" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D77" s="26" t="s">
+      <c r="D77" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E77" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F77" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G77" s="31">
+      <c r="E77" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F77" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G77" s="28">
         <v>23349.35</v>
       </c>
-      <c r="H77" s="31">
+      <c r="H77" s="28">
         <v>17500</v>
       </c>
-      <c r="I77" s="26"/>
-      <c r="J77" s="27"/>
-      <c r="K77" s="27"/>
-      <c r="L77" s="28"/>
-      <c r="M77" s="29"/>
-      <c r="N77" s="30"/>
-    </row>
-    <row r="78" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A78" s="26" t="s">
+      <c r="I77" s="5">
+        <v>1</v>
+      </c>
+      <c r="J77" s="14">
+        <f t="shared" si="6"/>
+        <v>23349.35</v>
+      </c>
+      <c r="K77" s="14">
+        <f t="shared" si="7"/>
+        <v>17500</v>
+      </c>
+      <c r="L77" s="25"/>
+      <c r="M77" s="26"/>
+      <c r="N77" s="27"/>
+    </row>
+    <row r="78" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A78" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B78" s="26" t="s">
+      <c r="B78" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="C78" s="26" t="s">
+      <c r="C78" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D78" s="26" t="s">
+      <c r="D78" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="E78" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F78" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G78" s="31">
+      <c r="E78" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F78" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G78" s="28">
         <v>15096.71</v>
       </c>
-      <c r="H78" s="31">
+      <c r="H78" s="28">
         <v>9100</v>
       </c>
-      <c r="I78" s="26"/>
-      <c r="J78" s="27"/>
-      <c r="K78" s="27"/>
-      <c r="L78" s="28"/>
-      <c r="M78" s="29"/>
-      <c r="N78" s="30"/>
-    </row>
-    <row r="79" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A79" s="26" t="s">
+      <c r="I78" s="5">
+        <v>1</v>
+      </c>
+      <c r="J78" s="14">
+        <f t="shared" si="6"/>
+        <v>15096.71</v>
+      </c>
+      <c r="K78" s="14">
+        <f t="shared" si="7"/>
+        <v>9100</v>
+      </c>
+      <c r="L78" s="25"/>
+      <c r="M78" s="26"/>
+      <c r="N78" s="27"/>
+    </row>
+    <row r="79" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A79" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B79" s="33" t="s">
+      <c r="B79" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="C79" s="26" t="s">
+      <c r="C79" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D79" s="26" t="s">
+      <c r="D79" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="E79" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F79" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G79" s="26">
+      <c r="E79" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F79" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G79" s="24">
         <v>328.65</v>
       </c>
-      <c r="H79" s="31">
+      <c r="H79" s="28">
         <v>21200</v>
       </c>
-      <c r="I79" s="26"/>
-      <c r="J79" s="27"/>
-      <c r="K79" s="27"/>
-      <c r="L79" s="28"/>
-      <c r="M79" s="29"/>
-      <c r="N79" s="30"/>
-    </row>
-    <row r="80" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A80" s="26" t="s">
+      <c r="I79" s="5">
+        <v>1</v>
+      </c>
+      <c r="J79" s="14">
+        <f t="shared" si="6"/>
+        <v>328.65</v>
+      </c>
+      <c r="K79" s="14">
+        <f t="shared" si="7"/>
+        <v>21200</v>
+      </c>
+      <c r="L79" s="25"/>
+      <c r="M79" s="26"/>
+      <c r="N79" s="27"/>
+    </row>
+    <row r="80" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A80" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B80" s="26" t="s">
+      <c r="B80" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="C80" s="26" t="s">
+      <c r="C80" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D80" s="26" t="s">
+      <c r="D80" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="E80" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F80" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G80" s="31">
+      <c r="E80" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F80" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G80" s="28">
         <v>39940.31</v>
       </c>
-      <c r="H80" s="31">
+      <c r="H80" s="28">
         <v>26973.19</v>
       </c>
-      <c r="I80" s="26"/>
-      <c r="J80" s="27"/>
-      <c r="K80" s="27"/>
-      <c r="L80" s="28"/>
-      <c r="M80" s="29"/>
-      <c r="N80" s="30"/>
-    </row>
-    <row r="81" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A81" s="26" t="s">
+      <c r="I80" s="5">
+        <v>1</v>
+      </c>
+      <c r="J80" s="14">
+        <f t="shared" si="6"/>
+        <v>39940.31</v>
+      </c>
+      <c r="K80" s="14">
+        <f t="shared" si="7"/>
+        <v>26973.19</v>
+      </c>
+      <c r="L80" s="25"/>
+      <c r="M80" s="26"/>
+      <c r="N80" s="27"/>
+    </row>
+    <row r="81" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A81" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B81" s="26" t="s">
+      <c r="B81" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C81" s="26" t="s">
+      <c r="C81" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D81" s="26" t="s">
+      <c r="D81" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E81" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F81" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G81" s="26">
+      <c r="E81" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F81" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G81" s="24">
         <v>822.89</v>
       </c>
-      <c r="H81" s="26">
+      <c r="H81" s="24">
         <v>822.89</v>
       </c>
-      <c r="I81" s="26"/>
-      <c r="J81" s="27"/>
-      <c r="K81" s="27"/>
-      <c r="L81" s="28"/>
-      <c r="M81" s="29"/>
-      <c r="N81" s="30"/>
-    </row>
-    <row r="82" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A82" s="26" t="s">
+      <c r="I81" s="5">
+        <v>1</v>
+      </c>
+      <c r="J81" s="14">
+        <f t="shared" si="6"/>
+        <v>822.89</v>
+      </c>
+      <c r="K81" s="14">
+        <f t="shared" si="7"/>
+        <v>822.89</v>
+      </c>
+      <c r="L81" s="25"/>
+      <c r="M81" s="26"/>
+      <c r="N81" s="27"/>
+    </row>
+    <row r="82" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A82" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B82" s="26" t="s">
+      <c r="B82" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C82" s="26" t="s">
+      <c r="C82" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D82" s="26" t="s">
+      <c r="D82" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E82" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F82" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G82" s="26">
+      <c r="E82" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F82" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G82" s="24">
         <v>5.37</v>
       </c>
-      <c r="H82" s="26">
+      <c r="H82" s="24">
         <v>5.37</v>
       </c>
-      <c r="I82" s="26"/>
-      <c r="J82" s="27"/>
-      <c r="K82" s="27"/>
-      <c r="L82" s="28"/>
-      <c r="M82" s="29"/>
-      <c r="N82" s="30"/>
-    </row>
-    <row r="83" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A83" s="26" t="s">
+      <c r="I82" s="5">
+        <v>1</v>
+      </c>
+      <c r="J82" s="14">
+        <f t="shared" si="6"/>
+        <v>5.37</v>
+      </c>
+      <c r="K82" s="14">
+        <f t="shared" si="7"/>
+        <v>5.37</v>
+      </c>
+      <c r="L82" s="25"/>
+      <c r="M82" s="26"/>
+      <c r="N82" s="27"/>
+    </row>
+    <row r="83" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A83" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B83" s="26" t="s">
+      <c r="B83" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C83" s="26" t="s">
+      <c r="C83" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D83" s="26" t="s">
+      <c r="D83" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="E83" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F83" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G83" s="31">
+      <c r="E83" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F83" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G83" s="28">
         <v>56444.42</v>
       </c>
-      <c r="H83" s="31">
+      <c r="H83" s="28">
         <v>42000</v>
       </c>
-      <c r="I83" s="26"/>
-      <c r="J83" s="27"/>
-      <c r="K83" s="27"/>
-      <c r="L83" s="28"/>
-      <c r="M83" s="29"/>
-      <c r="N83" s="30"/>
-    </row>
-    <row r="84" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A84" s="26" t="s">
+      <c r="I83" s="5">
+        <v>1</v>
+      </c>
+      <c r="J83" s="14">
+        <f t="shared" si="6"/>
+        <v>56444.42</v>
+      </c>
+      <c r="K83" s="14">
+        <f t="shared" si="7"/>
+        <v>42000</v>
+      </c>
+      <c r="L83" s="25"/>
+      <c r="M83" s="26"/>
+      <c r="N83" s="27"/>
+    </row>
+    <row r="84" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A84" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="B84" s="26" t="s">
+      <c r="B84" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="C84" s="26" t="s">
+      <c r="C84" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D84" s="26" t="s">
+      <c r="D84" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="E84" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F84" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G84" s="31">
+      <c r="E84" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F84" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G84" s="28">
         <v>1825.43</v>
       </c>
-      <c r="H84" s="31">
+      <c r="H84" s="28">
         <v>1500</v>
       </c>
-      <c r="I84" s="26"/>
-      <c r="J84" s="27"/>
-      <c r="K84" s="27"/>
-      <c r="L84" s="28"/>
-      <c r="M84" s="29"/>
-      <c r="N84" s="30"/>
-    </row>
-    <row r="85" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A85" s="26" t="s">
+      <c r="I84" s="5">
+        <v>1</v>
+      </c>
+      <c r="J84" s="14">
+        <f t="shared" si="6"/>
+        <v>1825.43</v>
+      </c>
+      <c r="K84" s="14">
+        <f t="shared" si="7"/>
+        <v>1500</v>
+      </c>
+      <c r="L84" s="25"/>
+      <c r="M84" s="26"/>
+      <c r="N84" s="27"/>
+    </row>
+    <row r="85" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A85" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="B85" s="26" t="s">
+      <c r="B85" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="C85" s="26" t="s">
+      <c r="C85" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D85" s="26" t="s">
+      <c r="D85" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="E85" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F85" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G85" s="31">
+      <c r="E85" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F85" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G85" s="28">
         <v>3451.7</v>
       </c>
-      <c r="H85" s="31">
+      <c r="H85" s="28">
         <v>1990</v>
       </c>
-      <c r="I85" s="26"/>
-      <c r="J85" s="27"/>
-      <c r="K85" s="27"/>
-      <c r="L85" s="28"/>
-      <c r="M85" s="29"/>
-      <c r="N85" s="30"/>
-    </row>
-    <row r="86" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A86" s="26" t="s">
+      <c r="I85" s="5">
+        <v>1</v>
+      </c>
+      <c r="J85" s="14">
+        <f t="shared" si="6"/>
+        <v>3451.7</v>
+      </c>
+      <c r="K85" s="14">
+        <f t="shared" si="7"/>
+        <v>1990</v>
+      </c>
+      <c r="L85" s="25"/>
+      <c r="M85" s="26"/>
+      <c r="N85" s="27"/>
+    </row>
+    <row r="86" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A86" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="B86" s="26" t="s">
+      <c r="B86" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C86" s="26" t="s">
+      <c r="C86" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D86" s="26" t="s">
+      <c r="D86" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="E86" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F86" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G86" s="31">
+      <c r="E86" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F86" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G86" s="28">
         <v>13073.77</v>
       </c>
-      <c r="H86" s="31">
+      <c r="H86" s="28">
         <v>10000</v>
       </c>
-      <c r="I86" s="26"/>
-      <c r="J86" s="27"/>
-      <c r="K86" s="27"/>
-      <c r="L86" s="28"/>
-      <c r="M86" s="29"/>
-      <c r="N86" s="30"/>
-    </row>
-    <row r="87" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A87" s="26" t="s">
+      <c r="I86" s="5">
+        <v>1</v>
+      </c>
+      <c r="J86" s="14">
+        <f t="shared" si="6"/>
+        <v>13073.77</v>
+      </c>
+      <c r="K86" s="14">
+        <f t="shared" si="7"/>
+        <v>10000</v>
+      </c>
+      <c r="L86" s="25"/>
+      <c r="M86" s="26"/>
+      <c r="N86" s="27"/>
+    </row>
+    <row r="87" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A87" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="B87" s="26" t="s">
+      <c r="B87" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C87" s="26" t="s">
+      <c r="C87" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D87" s="26" t="s">
+      <c r="D87" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E87" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F87" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G87" s="26">
+      <c r="E87" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F87" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G87" s="24">
         <v>12.1</v>
       </c>
-      <c r="H87" s="26">
+      <c r="H87" s="24">
         <v>12.1</v>
       </c>
-      <c r="I87" s="26"/>
-      <c r="J87" s="27"/>
-      <c r="K87" s="27"/>
-      <c r="L87" s="28"/>
-      <c r="M87" s="29"/>
-      <c r="N87" s="30"/>
-    </row>
-    <row r="88" spans="1:14" ht="22.15" customHeight="1">
-      <c r="A88" s="26" t="s">
+      <c r="I87" s="5">
+        <v>1</v>
+      </c>
+      <c r="J87" s="14">
+        <f t="shared" si="6"/>
+        <v>12.1</v>
+      </c>
+      <c r="K87" s="14">
+        <f t="shared" si="7"/>
+        <v>12.1</v>
+      </c>
+      <c r="L87" s="25"/>
+      <c r="M87" s="26"/>
+      <c r="N87" s="27"/>
+    </row>
+    <row r="88" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A88" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="B88" s="26" t="s">
+      <c r="B88" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C88" s="26" t="s">
+      <c r="C88" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="D88" s="26" t="s">
+      <c r="D88" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E88" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="F88" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="G88" s="26">
+      <c r="E88" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F88" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G88" s="24">
         <v>10.5</v>
       </c>
-      <c r="H88" s="26">
+      <c r="H88" s="24">
         <v>10.5</v>
       </c>
-      <c r="I88" s="26"/>
-      <c r="J88" s="27"/>
-      <c r="K88" s="27"/>
-      <c r="L88" s="28"/>
-      <c r="M88" s="29"/>
-      <c r="N88" s="30"/>
-    </row>
-    <row r="89" spans="1:14" ht="26.1" customHeight="1">
+      <c r="I88" s="5">
+        <v>1</v>
+      </c>
+      <c r="J88" s="14">
+        <f t="shared" si="6"/>
+        <v>10.5</v>
+      </c>
+      <c r="K88" s="14">
+        <f t="shared" si="7"/>
+        <v>10.5</v>
+      </c>
+      <c r="L88" s="25"/>
+      <c r="M88" s="26"/>
+      <c r="N88" s="27"/>
+    </row>
+    <row r="89" spans="1:14" ht="26.1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A89" s="18" t="s">
         <v>115</v>
       </c>
@@ -4821,25 +5124,24 @@
       </c>
       <c r="J89" s="19">
         <f>SUM(J5:J54)</f>
-        <v>1455675.1769999999</v>
+        <v>1872608.537</v>
       </c>
       <c r="K89" s="19">
         <f>SUM(K5:K54)</f>
-        <v>1388657.1629999999</v>
+        <v>1799825.0230000003</v>
       </c>
       <c r="L89" s="18" t="s">
         <v>0</v>
       </c>
       <c r="M89" s="19">
         <f>SUM(M5:M54)</f>
-        <v>67018.013999999981</v>
+        <v>72783.513999999996</v>
       </c>
       <c r="N89" s="20">
         <f>IF(SUM(K5:K54)&gt;0,SUM(M5:M54)/SUM(K5:K54),0)</f>
-        <v>4.8261022076332302E-2</v>
-      </c>
-    </row>
-    <row r="90" spans="1:14" ht="15"/>
+        <v>4.0439216629337853E-2</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
fix: Tasks are the single source of truth — stop listing completed meeting action items
Morning plan / urgent answers were pulling to-dos from raw meeting action items
(which never get marked done) AND from Open Tasks, so completed items reappeared.
Now meeting action items are context-only; OPEN TASKS is the authoritative,
completion-aware to-do list. Prompt updated to never list meeting items as tasks.
</commit_message>
<xml_diff>
--- a/notion-import-templates/3_Portfolio_Holdings.xlsx
+++ b/notion-import-templates/3_Portfolio_Holdings.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="385" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91AC5B45-519D-430C-A88A-1D180417C7FD}"/>
+  <xr:revisionPtr revIDLastSave="387" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32EC0601-B487-4E93-BB64-C48890131CE2}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4444,15 +4444,15 @@
         <v>20000</v>
       </c>
       <c r="I72" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J72" s="14">
         <f t="shared" si="6"/>
-        <v>25.6</v>
+        <v>102.4</v>
       </c>
       <c r="K72" s="14">
         <f t="shared" si="7"/>
-        <v>20000</v>
+        <v>80000</v>
       </c>
       <c r="L72" s="25"/>
       <c r="M72" s="26"/>
@@ -4484,15 +4484,15 @@
         <v>34.49</v>
       </c>
       <c r="I73" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J73" s="14">
         <f t="shared" si="6"/>
-        <v>34.49</v>
+        <v>137.96</v>
       </c>
       <c r="K73" s="14">
         <f t="shared" si="7"/>
-        <v>34.49</v>
+        <v>137.96</v>
       </c>
       <c r="L73" s="25"/>
       <c r="M73" s="26"/>

</xml_diff>

<commit_message>
ux: institution whitelist needs only domain (drop Contact Email field)
Domain is what drives email filtering, so the add form now asks only for
Company Name + Email Domain (accepts a full email or URL and extracts the
domain). Removed the Contact Email field and its state. Compose picker shows
the domain when no email is set.
</commit_message>
<xml_diff>
--- a/notion-import-templates/3_Portfolio_Holdings.xlsx
+++ b/notion-import-templates/3_Portfolio_Holdings.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30128"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="387" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32EC0601-B487-4E93-BB64-C48890131CE2}"/>
+  <xr:revisionPtr revIDLastSave="406" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBD1254D-601E-46B7-8142-E7D7D180ED1B}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -11,6 +11,9 @@
     <sheet name="📋 READ ME FIRST" sheetId="1" r:id="rId1"/>
     <sheet name="Portfolio Data Entry" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Portfolio Data Entry'!$A$1:$N$91</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -32,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="117">
   <si>
     <t/>
   </si>
@@ -379,6 +382,10 @@
   </si>
   <si>
     <t>JANICE QUEK KHANG WEN</t>
+  </si>
+  <si>
+    <t>1. AmHong Kong Tech Index Fund - MYR
+2.Manulife Investment Greater China Fund</t>
   </si>
   <si>
     <t>TOTAL</t>
@@ -392,7 +399,7 @@
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -610,7 +617,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -692,6 +699,10 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1032,14 +1043,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C29"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" ht="20.65" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:3" ht="20.65">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1050,7 +1061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1061,7 +1072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -1072,7 +1083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -1083,7 +1094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -1094,7 +1105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -1105,7 +1116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" ht="25.5">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -1116,7 +1127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" ht="25.5">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -1127,7 +1138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" ht="25.5">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1138,7 +1149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1149,7 +1160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -1160,7 +1171,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" ht="25.5">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -1171,7 +1182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1182,7 +1193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -1193,7 +1204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -1204,7 +1215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1215,7 +1226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>0</v>
       </c>
@@ -1226,7 +1237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -1237,7 +1248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -1248,7 +1259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1259,7 +1270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:3" ht="25.5">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -1270,7 +1281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:3" ht="25.5">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -1281,7 +1292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:3" ht="25.5">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -1292,7 +1303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:3" ht="25.5">
       <c r="A28" t="s">
         <v>0</v>
       </c>
@@ -1303,7 +1314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:3" ht="25.5">
       <c r="A29" t="s">
         <v>0</v>
       </c>
@@ -1322,11 +1333,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N89"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:N91"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="54.265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="54.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="29" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
@@ -1340,7 +1351,7 @@
     <col min="14" max="14" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" ht="28.15" customHeight="1">
       <c r="A1" s="31" t="s">
         <v>26</v>
       </c>
@@ -1358,7 +1369,7 @@
       <c r="M1" s="31"/>
       <c r="N1" s="31"/>
     </row>
-    <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="32" t="s">
         <v>27</v>
       </c>
@@ -1376,7 +1387,7 @@
       <c r="M2" s="32"/>
       <c r="N2" s="32"/>
     </row>
-    <row r="3" spans="1:14" ht="32.1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" ht="32.1" customHeight="1">
       <c r="A3" s="10" t="s">
         <v>28</v>
       </c>
@@ -1420,7 +1431,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" ht="28.15" customHeight="1">
       <c r="A4" s="13" t="s">
         <v>42</v>
       </c>
@@ -1464,7 +1475,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" ht="22.15" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>55</v>
       </c>
@@ -1510,7 +1521,7 @@
         <v>0.81413355794360354</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" ht="22.15" customHeight="1">
       <c r="A6" s="5" t="s">
         <v>61</v>
       </c>
@@ -1546,7 +1557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:14" ht="22.15" customHeight="1">
       <c r="A7" s="5" t="s">
         <v>63</v>
       </c>
@@ -1582,7 +1593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:14" ht="22.15" customHeight="1">
       <c r="A8" s="5" t="s">
         <v>64</v>
       </c>
@@ -1628,7 +1639,7 @@
         <v>0.31638285714285719</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:14" ht="22.15" customHeight="1">
       <c r="A9" s="5" t="s">
         <v>67</v>
       </c>
@@ -1674,7 +1685,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:14" ht="22.15" customHeight="1">
       <c r="A10" s="5" t="s">
         <v>55</v>
       </c>
@@ -1720,7 +1731,7 @@
         <v>2.115999999999996E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" ht="22.15" customHeight="1">
       <c r="A11" s="5" t="s">
         <v>55</v>
       </c>
@@ -1766,7 +1777,7 @@
         <v>0.70171076923076936</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:14" ht="22.15" customHeight="1">
       <c r="A12" s="5" t="s">
         <v>55</v>
       </c>
@@ -1812,7 +1823,7 @@
         <v>8.044813559322038E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" ht="22.15" customHeight="1">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -1858,7 +1869,7 @@
         <v>7.6937391304347846E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" ht="22.15" customHeight="1">
       <c r="A14" s="5" t="s">
         <v>55</v>
       </c>
@@ -1904,7 +1915,7 @@
         <v>0.23820344424635223</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:14" ht="22.15" customHeight="1">
       <c r="A15" s="5" t="s">
         <v>55</v>
       </c>
@@ -1950,7 +1961,7 @@
         <v>-3.4960866666666701E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" ht="22.15" customHeight="1">
       <c r="A16" s="5" t="s">
         <v>55</v>
       </c>
@@ -1996,7 +2007,7 @@
         <v>0.33413971962616829</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:14" ht="22.15" customHeight="1">
       <c r="A17" s="5" t="s">
         <v>61</v>
       </c>
@@ -2042,7 +2053,7 @@
         <v>0.75419066666666668</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:14" ht="22.15" customHeight="1">
       <c r="A18" s="5" t="s">
         <v>61</v>
       </c>
@@ -2088,7 +2099,7 @@
         <v>8.0448192771084337E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:14" ht="22.15" customHeight="1">
       <c r="A19" s="5" t="s">
         <v>61</v>
       </c>
@@ -2134,7 +2145,7 @@
         <v>4.9483352468427097E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:14" ht="22.15" customHeight="1">
       <c r="A20" s="5" t="s">
         <v>61</v>
       </c>
@@ -2180,7 +2191,7 @@
         <v>0.41930928987468363</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:14" ht="22.15" customHeight="1">
       <c r="A21" s="5" t="s">
         <v>61</v>
       </c>
@@ -2226,7 +2237,7 @@
         <v>8.5334109223917844E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:14" ht="22.15" customHeight="1">
       <c r="A22" s="5" t="s">
         <v>63</v>
       </c>
@@ -2272,7 +2283,7 @@
         <v>0.75419099999999994</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:14" ht="22.15" customHeight="1">
       <c r="A23" s="5" t="s">
         <v>63</v>
       </c>
@@ -2318,7 +2329,7 @@
         <v>8.0448473282442742E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:14" ht="22.15" customHeight="1">
       <c r="A24" s="5" t="s">
         <v>63</v>
       </c>
@@ -2364,7 +2375,7 @@
         <v>0.41841675268897716</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:14" ht="22.15" customHeight="1">
       <c r="A25" s="5" t="s">
         <v>63</v>
       </c>
@@ -2410,7 +2421,7 @@
         <v>8.4817043627442735E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:14" ht="22.15" customHeight="1">
       <c r="A26" s="5" t="s">
         <v>64</v>
       </c>
@@ -2456,7 +2467,7 @@
         <v>7.7633806146572185E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:14" ht="22.15" customHeight="1">
       <c r="A27" s="5" t="s">
         <v>64</v>
       </c>
@@ -2502,7 +2513,7 @@
         <v>5.2741735537189423E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:14" ht="22.15" customHeight="1">
       <c r="A28" s="5" t="s">
         <v>64</v>
       </c>
@@ -2548,7 +2559,7 @@
         <v>0.39329555555555556</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:14" ht="22.15" customHeight="1">
       <c r="A29" s="5" t="s">
         <v>64</v>
       </c>
@@ -2588,7 +2599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:14" ht="22.15" customHeight="1">
       <c r="A30" s="5" t="s">
         <v>67</v>
       </c>
@@ -2634,7 +2645,7 @@
         <v>0.15268291916376459</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:14" ht="22.15" customHeight="1">
       <c r="A31" s="5" t="s">
         <v>67</v>
       </c>
@@ -2680,7 +2691,7 @@
         <v>0.29576248974094027</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="25.5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:14" ht="25.5">
       <c r="A32" s="5" t="s">
         <v>83</v>
       </c>
@@ -2726,7 +2737,7 @@
         <v>-0.99778234042553182</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:14" ht="22.15" customHeight="1">
       <c r="A33" s="5" t="s">
         <v>83</v>
       </c>
@@ -2772,7 +2783,7 @@
         <v>0.2698421508733983</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:14" ht="22.15" customHeight="1">
       <c r="A34" s="5" t="s">
         <v>86</v>
       </c>
@@ -2818,7 +2829,7 @@
         <v>0.1016704587840358</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:14" ht="22.15" customHeight="1">
       <c r="A35" s="5" t="s">
         <v>86</v>
       </c>
@@ -2864,7 +2875,7 @@
         <v>0.18256140350877198</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:14" ht="22.15" customHeight="1">
       <c r="A36" s="5" t="s">
         <v>88</v>
       </c>
@@ -2910,7 +2921,7 @@
         <v>0.36689935589054251</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:14" ht="22.15" customHeight="1">
       <c r="A37" s="5" t="s">
         <v>90</v>
       </c>
@@ -2956,7 +2967,7 @@
         <v>-0.99959411764705874</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:14" ht="22.15" customHeight="1">
       <c r="A38" s="5" t="s">
         <v>90</v>
       </c>
@@ -3002,7 +3013,7 @@
         <v>-0.9997466647598422</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:14" ht="22.15" customHeight="1">
       <c r="A39" s="5" t="s">
         <v>92</v>
       </c>
@@ -3048,7 +3059,7 @@
         <v>0.35028333333333328</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:14" ht="22.15" customHeight="1">
       <c r="A40" s="5" t="s">
         <v>92</v>
       </c>
@@ -3094,7 +3105,7 @@
         <v>0.88331999999999988</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:14" ht="22.15" customHeight="1">
       <c r="A41" s="5" t="s">
         <v>92</v>
       </c>
@@ -3140,7 +3151,7 @@
         <v>-0.99992081967213109</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:14" ht="22.15" customHeight="1">
       <c r="A42" s="5" t="s">
         <v>94</v>
       </c>
@@ -3186,7 +3197,7 @@
         <v>7.7726666666666763E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:14" ht="22.15" customHeight="1">
       <c r="A43" s="5" t="s">
         <v>94</v>
       </c>
@@ -3232,7 +3243,7 @@
         <v>4.50014799154334E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:14" ht="22.15" customHeight="1">
       <c r="A44" s="5" t="s">
         <v>94</v>
       </c>
@@ -3278,7 +3289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:14" ht="22.15" customHeight="1">
       <c r="A45" s="5" t="s">
         <v>94</v>
       </c>
@@ -3324,7 +3335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:14" ht="22.15" customHeight="1">
       <c r="A46" s="5" t="s">
         <v>94</v>
       </c>
@@ -3370,7 +3381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:14" ht="22.15" customHeight="1">
       <c r="A47" s="5" t="s">
         <v>94</v>
       </c>
@@ -3416,7 +3427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:14" ht="22.15" customHeight="1">
       <c r="A48" s="5" t="s">
         <v>94</v>
       </c>
@@ -3462,7 +3473,7 @@
         <v>0.25449884761640745</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:14" ht="22.15" customHeight="1">
       <c r="A49" s="5" t="s">
         <v>94</v>
       </c>
@@ -3508,7 +3519,7 @@
         <v>0.24372296294294435</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:14" ht="22.15" customHeight="1">
       <c r="A50" s="5" t="s">
         <v>94</v>
       </c>
@@ -3554,7 +3565,7 @@
         <v>-5.1500000000000001E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:14" ht="22.15" customHeight="1">
       <c r="A51" s="5" t="s">
         <v>94</v>
       </c>
@@ -3600,7 +3611,7 @@
         <v>0.42390989282327485</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:14" ht="22.15" customHeight="1">
       <c r="A52" s="5" t="s">
         <v>94</v>
       </c>
@@ -3646,7 +3657,7 @@
         <v>0.33006799999999992</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:14" ht="22.15" customHeight="1">
       <c r="A53" s="5" t="s">
         <v>101</v>
       </c>
@@ -3692,7 +3703,7 @@
         <v>0.70702519379844964</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:14" ht="22.15" customHeight="1">
       <c r="A54" s="5" t="s">
         <v>101</v>
       </c>
@@ -3738,7 +3749,7 @@
         <v>0.11434999999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:14" ht="22.15" customHeight="1">
       <c r="A55" s="5" t="s">
         <v>101</v>
       </c>
@@ -3778,7 +3789,7 @@
       <c r="M55" s="26"/>
       <c r="N55" s="27"/>
     </row>
-    <row r="56" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:14" ht="22.15" customHeight="1">
       <c r="A56" s="5" t="s">
         <v>101</v>
       </c>
@@ -3818,7 +3829,7 @@
       <c r="M56" s="26"/>
       <c r="N56" s="27"/>
     </row>
-    <row r="57" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:14" ht="22.15" customHeight="1">
       <c r="A57" s="5" t="s">
         <v>101</v>
       </c>
@@ -3858,7 +3869,7 @@
       <c r="M57" s="26"/>
       <c r="N57" s="27"/>
     </row>
-    <row r="58" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:14" ht="22.15" customHeight="1">
       <c r="A58" s="5" t="s">
         <v>101</v>
       </c>
@@ -3898,7 +3909,7 @@
       <c r="M58" s="26"/>
       <c r="N58" s="27"/>
     </row>
-    <row r="59" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:14" ht="22.15" customHeight="1">
       <c r="A59" s="24" t="s">
         <v>104</v>
       </c>
@@ -3938,7 +3949,7 @@
       <c r="M59" s="26"/>
       <c r="N59" s="27"/>
     </row>
-    <row r="60" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:14" ht="22.15" customHeight="1">
       <c r="A60" s="24" t="s">
         <v>104</v>
       </c>
@@ -3978,7 +3989,7 @@
       <c r="M60" s="26"/>
       <c r="N60" s="27"/>
     </row>
-    <row r="61" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:14" ht="22.15" customHeight="1">
       <c r="A61" s="24" t="s">
         <v>104</v>
       </c>
@@ -4018,7 +4029,7 @@
       <c r="M61" s="26"/>
       <c r="N61" s="27"/>
     </row>
-    <row r="62" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:14" ht="22.15" customHeight="1">
       <c r="A62" s="24" t="s">
         <v>104</v>
       </c>
@@ -4058,7 +4069,7 @@
       <c r="M62" s="26"/>
       <c r="N62" s="27"/>
     </row>
-    <row r="63" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:14" ht="22.15" customHeight="1">
       <c r="A63" s="24" t="s">
         <v>104</v>
       </c>
@@ -4098,7 +4109,7 @@
       <c r="M63" s="26"/>
       <c r="N63" s="27"/>
     </row>
-    <row r="64" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:14" ht="22.15" customHeight="1">
       <c r="A64" s="24" t="s">
         <v>106</v>
       </c>
@@ -4138,7 +4149,7 @@
       <c r="M64" s="26"/>
       <c r="N64" s="27"/>
     </row>
-    <row r="65" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:14" ht="22.15" customHeight="1">
       <c r="A65" s="24" t="s">
         <v>106</v>
       </c>
@@ -4178,7 +4189,7 @@
       <c r="M65" s="26"/>
       <c r="N65" s="27"/>
     </row>
-    <row r="66" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:14" ht="22.15" customHeight="1">
       <c r="A66" s="24" t="s">
         <v>106</v>
       </c>
@@ -4218,7 +4229,7 @@
       <c r="M66" s="26"/>
       <c r="N66" s="27"/>
     </row>
-    <row r="67" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:14" ht="22.15" customHeight="1">
       <c r="A67" s="24" t="s">
         <v>109</v>
       </c>
@@ -4258,7 +4269,7 @@
       <c r="M67" s="26"/>
       <c r="N67" s="27"/>
     </row>
-    <row r="68" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:14" ht="22.15" customHeight="1">
       <c r="A68" s="24" t="s">
         <v>109</v>
       </c>
@@ -4298,7 +4309,7 @@
       <c r="M68" s="26"/>
       <c r="N68" s="27"/>
     </row>
-    <row r="69" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:14" ht="22.15" customHeight="1">
       <c r="A69" s="24" t="s">
         <v>109</v>
       </c>
@@ -4338,7 +4349,7 @@
       <c r="M69" s="26"/>
       <c r="N69" s="27"/>
     </row>
-    <row r="70" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:14" ht="22.15" customHeight="1">
       <c r="A70" s="24" t="s">
         <v>110</v>
       </c>
@@ -4378,7 +4389,7 @@
       <c r="M70" s="26"/>
       <c r="N70" s="27"/>
     </row>
-    <row r="71" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:14" ht="22.15" customHeight="1">
       <c r="A71" s="24" t="s">
         <v>110</v>
       </c>
@@ -4418,7 +4429,7 @@
       <c r="M71" s="26"/>
       <c r="N71" s="27"/>
     </row>
-    <row r="72" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:14" ht="22.15" customHeight="1">
       <c r="A72" s="24" t="s">
         <v>110</v>
       </c>
@@ -4458,7 +4469,7 @@
       <c r="M72" s="26"/>
       <c r="N72" s="27"/>
     </row>
-    <row r="73" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:14" ht="22.15" customHeight="1">
       <c r="A73" s="24" t="s">
         <v>110</v>
       </c>
@@ -4498,7 +4509,7 @@
       <c r="M73" s="26"/>
       <c r="N73" s="27"/>
     </row>
-    <row r="74" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:14" ht="22.15" customHeight="1">
       <c r="A74" s="24" t="s">
         <v>110</v>
       </c>
@@ -4538,7 +4549,7 @@
       <c r="M74" s="26"/>
       <c r="N74" s="27"/>
     </row>
-    <row r="75" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:14" ht="22.15" customHeight="1">
       <c r="A75" s="24" t="s">
         <v>112</v>
       </c>
@@ -4574,7 +4585,7 @@
       <c r="M75" s="26"/>
       <c r="N75" s="27"/>
     </row>
-    <row r="76" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:14" ht="22.15" customHeight="1">
       <c r="A76" s="24" t="s">
         <v>112</v>
       </c>
@@ -4614,7 +4625,7 @@
       <c r="M76" s="26"/>
       <c r="N76" s="27"/>
     </row>
-    <row r="77" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:14" ht="22.15" customHeight="1">
       <c r="A77" s="24" t="s">
         <v>112</v>
       </c>
@@ -4654,7 +4665,7 @@
       <c r="M77" s="26"/>
       <c r="N77" s="27"/>
     </row>
-    <row r="78" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:14" ht="22.15" customHeight="1">
       <c r="A78" s="24" t="s">
         <v>113</v>
       </c>
@@ -4694,7 +4705,7 @@
       <c r="M78" s="26"/>
       <c r="N78" s="27"/>
     </row>
-    <row r="79" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:14" ht="22.15" customHeight="1">
       <c r="A79" s="24" t="s">
         <v>113</v>
       </c>
@@ -4734,7 +4745,7 @@
       <c r="M79" s="26"/>
       <c r="N79" s="27"/>
     </row>
-    <row r="80" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:14" ht="22.15" customHeight="1">
       <c r="A80" s="24" t="s">
         <v>113</v>
       </c>
@@ -4774,7 +4785,7 @@
       <c r="M80" s="26"/>
       <c r="N80" s="27"/>
     </row>
-    <row r="81" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:14" ht="22.15" customHeight="1">
       <c r="A81" s="24" t="s">
         <v>113</v>
       </c>
@@ -4814,7 +4825,7 @@
       <c r="M81" s="26"/>
       <c r="N81" s="27"/>
     </row>
-    <row r="82" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:14" ht="22.15" customHeight="1">
       <c r="A82" s="24" t="s">
         <v>113</v>
       </c>
@@ -4854,7 +4865,7 @@
       <c r="M82" s="26"/>
       <c r="N82" s="27"/>
     </row>
-    <row r="83" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:14" ht="22.15" customHeight="1">
       <c r="A83" s="24" t="s">
         <v>113</v>
       </c>
@@ -4894,7 +4905,7 @@
       <c r="M83" s="26"/>
       <c r="N83" s="27"/>
     </row>
-    <row r="84" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:14" ht="22.15" customHeight="1">
       <c r="A84" s="24" t="s">
         <v>114</v>
       </c>
@@ -4934,7 +4945,7 @@
       <c r="M84" s="26"/>
       <c r="N84" s="27"/>
     </row>
-    <row r="85" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:14" ht="22.15" customHeight="1">
       <c r="A85" s="24" t="s">
         <v>114</v>
       </c>
@@ -4974,7 +4985,7 @@
       <c r="M85" s="26"/>
       <c r="N85" s="27"/>
     </row>
-    <row r="86" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:14" ht="22.15" customHeight="1">
       <c r="A86" s="24" t="s">
         <v>114</v>
       </c>
@@ -5014,7 +5025,7 @@
       <c r="M86" s="26"/>
       <c r="N86" s="27"/>
     </row>
-    <row r="87" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:14" ht="22.15" customHeight="1">
       <c r="A87" s="24" t="s">
         <v>114</v>
       </c>
@@ -5054,7 +5065,7 @@
       <c r="M87" s="26"/>
       <c r="N87" s="27"/>
     </row>
-    <row r="88" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:14" ht="22.15" customHeight="1">
       <c r="A88" s="24" t="s">
         <v>114</v>
       </c>
@@ -5094,70 +5105,149 @@
       <c r="M88" s="26"/>
       <c r="N88" s="27"/>
     </row>
-    <row r="89" spans="1:14" ht="26.1" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A89" s="18" t="s">
+    <row r="89" spans="1:14" ht="22.15" customHeight="1">
+      <c r="A89" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B89" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="B89" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="C89" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="D89" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="E89" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="F89" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="G89" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="H89" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="I89" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="J89" s="19">
+      <c r="C89" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="D89" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E89" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F89" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G89" s="28">
+        <v>23812.5</v>
+      </c>
+      <c r="H89" s="28">
+        <v>15000</v>
+      </c>
+      <c r="I89" s="33"/>
+      <c r="J89" s="34"/>
+      <c r="K89" s="34"/>
+      <c r="L89" s="25"/>
+      <c r="M89" s="26"/>
+      <c r="N89" s="27"/>
+    </row>
+    <row r="90" spans="1:14" ht="22.15" customHeight="1">
+      <c r="A90" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B90" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C90" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="D90" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E90" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F90" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G90" s="28">
+        <v>11943.34</v>
+      </c>
+      <c r="H90" s="28">
+        <v>11943.34</v>
+      </c>
+      <c r="I90" s="33"/>
+      <c r="J90" s="34"/>
+      <c r="K90" s="34"/>
+      <c r="L90" s="25"/>
+      <c r="M90" s="26"/>
+      <c r="N90" s="27"/>
+    </row>
+    <row r="91" spans="1:14" ht="26.1" customHeight="1">
+      <c r="A91" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="B91" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C91" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="D91" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="E91" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="F91" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G91" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="H91" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="I91" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="J91" s="19">
         <f>SUM(J5:J54)</f>
         <v>1872608.537</v>
       </c>
-      <c r="K89" s="19">
+      <c r="K91" s="19">
         <f>SUM(K5:K54)</f>
         <v>1799825.0230000003</v>
       </c>
-      <c r="L89" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="M89" s="19">
+      <c r="L91" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="M91" s="19">
         <f>SUM(M5:M54)</f>
         <v>72783.513999999996</v>
       </c>
-      <c r="N89" s="20">
+      <c r="N91" s="20">
         <f>IF(SUM(K5:K54)&gt;0,SUM(M5:M54)/SUM(K5:K54),0)</f>
         <v>4.0439216629337853E-2</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:N91" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="0" showButton="0"/>
+    <filterColumn colId="1" showButton="0"/>
+    <filterColumn colId="2" showButton="0"/>
+    <filterColumn colId="3" showButton="0"/>
+    <filterColumn colId="4" showButton="0"/>
+    <filterColumn colId="5" showButton="0"/>
+    <filterColumn colId="6" showButton="0"/>
+    <filterColumn colId="7" showButton="0"/>
+    <filterColumn colId="8" showButton="0"/>
+    <filterColumn colId="9" showButton="0"/>
+    <filterColumn colId="10" showButton="0"/>
+    <filterColumn colId="11" showButton="0"/>
+    <filterColumn colId="12" showButton="0"/>
+  </autoFilter>
   <mergeCells count="2">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A2:N2"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: EPF | Unit Trust | Fixed Deposit | Stocks | Bonds" sqref="C5:C88" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: EPF | Unit Trust | Fixed Deposit | Stocks | Bonds" sqref="C5:C90" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"EPF,Unit Trust,Fixed Deposit,Stocks,Bonds"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Active | Matured | Redeemed | Pending" sqref="E5:E88" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Active | Matured | Redeemed | Pending" sqref="E5:E90" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Active,Matured,Redeemed,Pending"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: MYR | USD | SGD | GBP | EUR | AUD | HKD | JPY | CNY" sqref="F5:F88" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: MYR | USD | SGD | GBP | EUR | AUD | HKD | JPY | CNY" sqref="F5:F90" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"MYR,USD,SGD,GBP,EUR,AUD,HKD,JPY,CNY"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="L5:L88" xr:uid="{00000000-0002-0000-0100-000003000000}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="L5:L90" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>TRUE</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
ux: Insurance table — dedicated Life/TPD, CI, Accident columns
Replaced the single 'Sum Assured' column (and the cramped cover-amounts text
under Benefits) with three independent coverage columns:
  Life / TPD  (= sum assured, since they're the same)  · CI · Accident
Each shows the amount (or — when zero), with column subtotals. Medical class
moved to the policy detail line. Removed now-unused BenefitPill/benefit colours.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/notion-import-templates/3_Portfolio_Holdings.xlsx
+++ b/notion-import-templates/3_Portfolio_Holdings.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="406" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBD1254D-601E-46B7-8142-E7D7D180ED1B}"/>
+  <xr:revisionPtr revIDLastSave="407" documentId="13_ncr:1_{52A364DC-9654-41CE-AD41-F2E07BC9A8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12FAB1C0-D45F-4AAC-9036-59FF42C83AD7}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12,7 +12,7 @@
     <sheet name="Portfolio Data Entry" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Portfolio Data Entry'!$A$1:$N$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Portfolio Data Entry'!$A$1:$N$92</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="117">
   <si>
     <t/>
   </si>
@@ -399,7 +399,7 @@
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -617,7 +617,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -693,16 +693,13 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1043,14 +1040,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:C29"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" ht="20.65">
+    <row r="2" spans="1:3" ht="20.65" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1061,7 +1058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -1072,7 +1069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -1083,7 +1080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -1094,7 +1091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -1105,7 +1102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -1116,7 +1113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="25.5">
+    <row r="9" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -1127,7 +1124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="25.5">
+    <row r="10" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -1138,7 +1135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="25.5">
+    <row r="11" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -1149,7 +1146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -1160,7 +1157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -1171,7 +1168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="25.5">
+    <row r="14" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -1182,7 +1179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -1193,7 +1190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>0</v>
       </c>
@@ -1204,7 +1201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>0</v>
       </c>
@@ -1215,7 +1212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>0</v>
       </c>
@@ -1226,7 +1223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>0</v>
       </c>
@@ -1237,7 +1234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>0</v>
       </c>
@@ -1248,7 +1245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -1259,7 +1256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -1270,7 +1267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="25.5">
+    <row r="25" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>0</v>
       </c>
@@ -1281,7 +1278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="25.5">
+    <row r="26" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>0</v>
       </c>
@@ -1292,7 +1289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="25.5">
+    <row r="27" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>0</v>
       </c>
@@ -1303,7 +1300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="25.5">
+    <row r="28" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>0</v>
       </c>
@@ -1314,7 +1311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="25.5">
+    <row r="29" spans="1:3" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>0</v>
       </c>
@@ -1333,11 +1330,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N91"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:N92"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="54.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="54.265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="29" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
@@ -1351,43 +1348,43 @@
     <col min="14" max="14" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28.15" customHeight="1">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:14" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-    </row>
-    <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1">
-      <c r="A2" s="32" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
+      <c r="L1" s="32"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="32"/>
+    </row>
+    <row r="2" spans="1:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="33" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-    </row>
-    <row r="3" spans="1:14" ht="32.1" customHeight="1">
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+    </row>
+    <row r="3" spans="1:14" ht="32.1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="10" t="s">
         <v>28</v>
       </c>
@@ -1431,7 +1428,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="28.15" customHeight="1">
+    <row r="4" spans="1:14" ht="28.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="13" t="s">
         <v>42</v>
       </c>
@@ -1475,7 +1472,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="22.15" customHeight="1">
+    <row r="5" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="5" t="s">
         <v>55</v>
       </c>
@@ -1521,7 +1518,7 @@
         <v>0.81413355794360354</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="22.15" customHeight="1">
+    <row r="6" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="5" t="s">
         <v>61</v>
       </c>
@@ -1557,7 +1554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="22.15" customHeight="1">
+    <row r="7" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="5" t="s">
         <v>63</v>
       </c>
@@ -1593,7 +1590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="22.15" customHeight="1">
+    <row r="8" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="5" t="s">
         <v>64</v>
       </c>
@@ -1639,7 +1636,7 @@
         <v>0.31638285714285719</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="22.15" customHeight="1">
+    <row r="9" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="5" t="s">
         <v>67</v>
       </c>
@@ -1685,7 +1682,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="22.15" customHeight="1">
+    <row r="10" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="5" t="s">
         <v>55</v>
       </c>
@@ -1731,7 +1728,7 @@
         <v>2.115999999999996E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="22.15" customHeight="1">
+    <row r="11" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="5" t="s">
         <v>55</v>
       </c>
@@ -1777,7 +1774,7 @@
         <v>0.70171076923076936</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="22.15" customHeight="1">
+    <row r="12" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="5" t="s">
         <v>55</v>
       </c>
@@ -1823,7 +1820,7 @@
         <v>8.044813559322038E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="22.15" customHeight="1">
+    <row r="13" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="5" t="s">
         <v>55</v>
       </c>
@@ -1869,7 +1866,7 @@
         <v>7.6937391304347846E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="22.15" customHeight="1">
+    <row r="14" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
         <v>55</v>
       </c>
@@ -1915,7 +1912,7 @@
         <v>0.23820344424635223</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="22.15" customHeight="1">
+    <row r="15" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
         <v>55</v>
       </c>
@@ -1961,7 +1958,7 @@
         <v>-3.4960866666666701E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="22.15" customHeight="1">
+    <row r="16" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="5" t="s">
         <v>55</v>
       </c>
@@ -2007,7 +2004,7 @@
         <v>0.33413971962616829</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="22.15" customHeight="1">
+    <row r="17" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="5" t="s">
         <v>61</v>
       </c>
@@ -2053,7 +2050,7 @@
         <v>0.75419066666666668</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="22.15" customHeight="1">
+    <row r="18" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="5" t="s">
         <v>61</v>
       </c>
@@ -2099,7 +2096,7 @@
         <v>8.0448192771084337E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="22.15" customHeight="1">
+    <row r="19" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="5" t="s">
         <v>61</v>
       </c>
@@ -2145,7 +2142,7 @@
         <v>4.9483352468427097E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="22.15" customHeight="1">
+    <row r="20" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="5" t="s">
         <v>61</v>
       </c>
@@ -2191,7 +2188,7 @@
         <v>0.41930928987468363</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="22.15" customHeight="1">
+    <row r="21" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="5" t="s">
         <v>61</v>
       </c>
@@ -2237,7 +2234,7 @@
         <v>8.5334109223917844E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="22.15" customHeight="1">
+    <row r="22" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="5" t="s">
         <v>63</v>
       </c>
@@ -2283,7 +2280,7 @@
         <v>0.75419099999999994</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="22.15" customHeight="1">
+    <row r="23" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="5" t="s">
         <v>63</v>
       </c>
@@ -2329,7 +2326,7 @@
         <v>8.0448473282442742E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="22.15" customHeight="1">
+    <row r="24" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="5" t="s">
         <v>63</v>
       </c>
@@ -2375,7 +2372,7 @@
         <v>0.41841675268897716</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="22.15" customHeight="1">
+    <row r="25" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="5" t="s">
         <v>63</v>
       </c>
@@ -2421,7 +2418,7 @@
         <v>8.4817043627442735E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="22.15" customHeight="1">
+    <row r="26" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="5" t="s">
         <v>64</v>
       </c>
@@ -2467,7 +2464,7 @@
         <v>7.7633806146572185E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="22.15" customHeight="1">
+    <row r="27" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="5" t="s">
         <v>64</v>
       </c>
@@ -2513,7 +2510,7 @@
         <v>5.2741735537189423E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="22.15" customHeight="1">
+    <row r="28" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="5" t="s">
         <v>64</v>
       </c>
@@ -2559,7 +2556,7 @@
         <v>0.39329555555555556</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="22.15" customHeight="1">
+    <row r="29" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="5" t="s">
         <v>64</v>
       </c>
@@ -2599,7 +2596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="22.15" customHeight="1">
+    <row r="30" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="5" t="s">
         <v>67</v>
       </c>
@@ -2645,7 +2642,7 @@
         <v>0.15268291916376459</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="22.15" customHeight="1">
+    <row r="31" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="5" t="s">
         <v>67</v>
       </c>
@@ -2691,7 +2688,7 @@
         <v>0.29576248974094027</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="25.5">
+    <row r="32" spans="1:14" ht="25.5" x14ac:dyDescent="0.45">
       <c r="A32" s="5" t="s">
         <v>83</v>
       </c>
@@ -2737,7 +2734,7 @@
         <v>-0.99778234042553182</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="22.15" customHeight="1">
+    <row r="33" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="5" t="s">
         <v>83</v>
       </c>
@@ -2783,7 +2780,7 @@
         <v>0.2698421508733983</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="22.15" customHeight="1">
+    <row r="34" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="5" t="s">
         <v>86</v>
       </c>
@@ -2829,7 +2826,7 @@
         <v>0.1016704587840358</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="22.15" customHeight="1">
+    <row r="35" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="5" t="s">
         <v>86</v>
       </c>
@@ -2875,7 +2872,7 @@
         <v>0.18256140350877198</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="22.15" customHeight="1">
+    <row r="36" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="5" t="s">
         <v>88</v>
       </c>
@@ -2921,7 +2918,7 @@
         <v>0.36689935589054251</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="22.15" customHeight="1">
+    <row r="37" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="5" t="s">
         <v>90</v>
       </c>
@@ -2967,7 +2964,7 @@
         <v>-0.99959411764705874</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="22.15" customHeight="1">
+    <row r="38" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="5" t="s">
         <v>90</v>
       </c>
@@ -3013,7 +3010,7 @@
         <v>-0.9997466647598422</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="22.15" customHeight="1">
+    <row r="39" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="5" t="s">
         <v>92</v>
       </c>
@@ -3059,7 +3056,7 @@
         <v>0.35028333333333328</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="22.15" customHeight="1">
+    <row r="40" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="5" t="s">
         <v>92</v>
       </c>
@@ -3105,7 +3102,7 @@
         <v>0.88331999999999988</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="22.15" customHeight="1">
+    <row r="41" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="5" t="s">
         <v>92</v>
       </c>
@@ -3151,7 +3148,7 @@
         <v>-0.99992081967213109</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="22.15" customHeight="1">
+    <row r="42" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="5" t="s">
         <v>94</v>
       </c>
@@ -3197,7 +3194,7 @@
         <v>7.7726666666666763E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="22.15" customHeight="1">
+    <row r="43" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="5" t="s">
         <v>94</v>
       </c>
@@ -3243,7 +3240,7 @@
         <v>4.50014799154334E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="22.15" customHeight="1">
+    <row r="44" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="5" t="s">
         <v>94</v>
       </c>
@@ -3289,7 +3286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="22.15" customHeight="1">
+    <row r="45" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="5" t="s">
         <v>94</v>
       </c>
@@ -3335,7 +3332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="22.15" customHeight="1">
+    <row r="46" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="5" t="s">
         <v>94</v>
       </c>
@@ -3381,7 +3378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="22.15" customHeight="1">
+    <row r="47" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="5" t="s">
         <v>94</v>
       </c>
@@ -3427,7 +3424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="22.15" customHeight="1">
+    <row r="48" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="5" t="s">
         <v>94</v>
       </c>
@@ -3473,7 +3470,7 @@
         <v>0.25449884761640745</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="22.15" customHeight="1">
+    <row r="49" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="5" t="s">
         <v>94</v>
       </c>
@@ -3519,7 +3516,7 @@
         <v>0.24372296294294435</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="22.15" customHeight="1">
+    <row r="50" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="5" t="s">
         <v>94</v>
       </c>
@@ -3565,7 +3562,7 @@
         <v>-5.1500000000000001E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="22.15" customHeight="1">
+    <row r="51" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="5" t="s">
         <v>94</v>
       </c>
@@ -3611,7 +3608,7 @@
         <v>0.42390989282327485</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="22.15" customHeight="1">
+    <row r="52" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="5" t="s">
         <v>94</v>
       </c>
@@ -3657,7 +3654,7 @@
         <v>0.33006799999999992</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="22.15" customHeight="1">
+    <row r="53" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="5" t="s">
         <v>101</v>
       </c>
@@ -3703,7 +3700,7 @@
         <v>0.70702519379844964</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="22.15" customHeight="1">
+    <row r="54" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="5" t="s">
         <v>101</v>
       </c>
@@ -3749,7 +3746,7 @@
         <v>0.11434999999999999</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="22.15" customHeight="1">
+    <row r="55" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="5" t="s">
         <v>101</v>
       </c>
@@ -3789,7 +3786,7 @@
       <c r="M55" s="26"/>
       <c r="N55" s="27"/>
     </row>
-    <row r="56" spans="1:14" ht="22.15" customHeight="1">
+    <row r="56" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="5" t="s">
         <v>101</v>
       </c>
@@ -3829,7 +3826,7 @@
       <c r="M56" s="26"/>
       <c r="N56" s="27"/>
     </row>
-    <row r="57" spans="1:14" ht="22.15" customHeight="1">
+    <row r="57" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="5" t="s">
         <v>101</v>
       </c>
@@ -3869,7 +3866,7 @@
       <c r="M57" s="26"/>
       <c r="N57" s="27"/>
     </row>
-    <row r="58" spans="1:14" ht="22.15" customHeight="1">
+    <row r="58" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="5" t="s">
         <v>101</v>
       </c>
@@ -3909,7 +3906,7 @@
       <c r="M58" s="26"/>
       <c r="N58" s="27"/>
     </row>
-    <row r="59" spans="1:14" ht="22.15" customHeight="1">
+    <row r="59" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="24" t="s">
         <v>104</v>
       </c>
@@ -3949,7 +3946,7 @@
       <c r="M59" s="26"/>
       <c r="N59" s="27"/>
     </row>
-    <row r="60" spans="1:14" ht="22.15" customHeight="1">
+    <row r="60" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="24" t="s">
         <v>104</v>
       </c>
@@ -3989,7 +3986,7 @@
       <c r="M60" s="26"/>
       <c r="N60" s="27"/>
     </row>
-    <row r="61" spans="1:14" ht="22.15" customHeight="1">
+    <row r="61" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="24" t="s">
         <v>104</v>
       </c>
@@ -4029,7 +4026,7 @@
       <c r="M61" s="26"/>
       <c r="N61" s="27"/>
     </row>
-    <row r="62" spans="1:14" ht="22.15" customHeight="1">
+    <row r="62" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="24" t="s">
         <v>104</v>
       </c>
@@ -4069,7 +4066,7 @@
       <c r="M62" s="26"/>
       <c r="N62" s="27"/>
     </row>
-    <row r="63" spans="1:14" ht="22.15" customHeight="1">
+    <row r="63" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A63" s="24" t="s">
         <v>104</v>
       </c>
@@ -4109,7 +4106,7 @@
       <c r="M63" s="26"/>
       <c r="N63" s="27"/>
     </row>
-    <row r="64" spans="1:14" ht="22.15" customHeight="1">
+    <row r="64" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="24" t="s">
         <v>106</v>
       </c>
@@ -4149,7 +4146,7 @@
       <c r="M64" s="26"/>
       <c r="N64" s="27"/>
     </row>
-    <row r="65" spans="1:14" ht="22.15" customHeight="1">
+    <row r="65" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A65" s="24" t="s">
         <v>106</v>
       </c>
@@ -4189,7 +4186,7 @@
       <c r="M65" s="26"/>
       <c r="N65" s="27"/>
     </row>
-    <row r="66" spans="1:14" ht="22.15" customHeight="1">
+    <row r="66" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A66" s="24" t="s">
         <v>106</v>
       </c>
@@ -4229,7 +4226,7 @@
       <c r="M66" s="26"/>
       <c r="N66" s="27"/>
     </row>
-    <row r="67" spans="1:14" ht="22.15" customHeight="1">
+    <row r="67" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" s="24" t="s">
         <v>109</v>
       </c>
@@ -4269,7 +4266,7 @@
       <c r="M67" s="26"/>
       <c r="N67" s="27"/>
     </row>
-    <row r="68" spans="1:14" ht="22.15" customHeight="1">
+    <row r="68" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="24" t="s">
         <v>109</v>
       </c>
@@ -4309,7 +4306,7 @@
       <c r="M68" s="26"/>
       <c r="N68" s="27"/>
     </row>
-    <row r="69" spans="1:14" ht="22.15" customHeight="1">
+    <row r="69" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="24" t="s">
         <v>109</v>
       </c>
@@ -4349,7 +4346,7 @@
       <c r="M69" s="26"/>
       <c r="N69" s="27"/>
     </row>
-    <row r="70" spans="1:14" ht="22.15" customHeight="1">
+    <row r="70" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="24" t="s">
         <v>110</v>
       </c>
@@ -4389,7 +4386,7 @@
       <c r="M70" s="26"/>
       <c r="N70" s="27"/>
     </row>
-    <row r="71" spans="1:14" ht="22.15" customHeight="1">
+    <row r="71" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="24" t="s">
         <v>110</v>
       </c>
@@ -4429,7 +4426,7 @@
       <c r="M71" s="26"/>
       <c r="N71" s="27"/>
     </row>
-    <row r="72" spans="1:14" ht="22.15" customHeight="1">
+    <row r="72" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="24" t="s">
         <v>110</v>
       </c>
@@ -4469,7 +4466,7 @@
       <c r="M72" s="26"/>
       <c r="N72" s="27"/>
     </row>
-    <row r="73" spans="1:14" ht="22.15" customHeight="1">
+    <row r="73" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="24" t="s">
         <v>110</v>
       </c>
@@ -4509,7 +4506,7 @@
       <c r="M73" s="26"/>
       <c r="N73" s="27"/>
     </row>
-    <row r="74" spans="1:14" ht="22.15" customHeight="1">
+    <row r="74" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A74" s="24" t="s">
         <v>110</v>
       </c>
@@ -4549,7 +4546,7 @@
       <c r="M74" s="26"/>
       <c r="N74" s="27"/>
     </row>
-    <row r="75" spans="1:14" ht="22.15" customHeight="1">
+    <row r="75" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="24" t="s">
         <v>112</v>
       </c>
@@ -4585,7 +4582,7 @@
       <c r="M75" s="26"/>
       <c r="N75" s="27"/>
     </row>
-    <row r="76" spans="1:14" ht="22.15" customHeight="1">
+    <row r="76" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="24" t="s">
         <v>112</v>
       </c>
@@ -4625,7 +4622,7 @@
       <c r="M76" s="26"/>
       <c r="N76" s="27"/>
     </row>
-    <row r="77" spans="1:14" ht="22.15" customHeight="1">
+    <row r="77" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A77" s="24" t="s">
         <v>112</v>
       </c>
@@ -4665,7 +4662,7 @@
       <c r="M77" s="26"/>
       <c r="N77" s="27"/>
     </row>
-    <row r="78" spans="1:14" ht="22.15" customHeight="1">
+    <row r="78" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" s="24" t="s">
         <v>113</v>
       </c>
@@ -4705,7 +4702,7 @@
       <c r="M78" s="26"/>
       <c r="N78" s="27"/>
     </row>
-    <row r="79" spans="1:14" ht="22.15" customHeight="1">
+    <row r="79" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A79" s="24" t="s">
         <v>113</v>
       </c>
@@ -4745,7 +4742,7 @@
       <c r="M79" s="26"/>
       <c r="N79" s="27"/>
     </row>
-    <row r="80" spans="1:14" ht="22.15" customHeight="1">
+    <row r="80" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A80" s="24" t="s">
         <v>113</v>
       </c>
@@ -4785,7 +4782,7 @@
       <c r="M80" s="26"/>
       <c r="N80" s="27"/>
     </row>
-    <row r="81" spans="1:14" ht="22.15" customHeight="1">
+    <row r="81" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A81" s="24" t="s">
         <v>113</v>
       </c>
@@ -4825,7 +4822,7 @@
       <c r="M81" s="26"/>
       <c r="N81" s="27"/>
     </row>
-    <row r="82" spans="1:14" ht="22.15" customHeight="1">
+    <row r="82" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A82" s="24" t="s">
         <v>113</v>
       </c>
@@ -4865,7 +4862,7 @@
       <c r="M82" s="26"/>
       <c r="N82" s="27"/>
     </row>
-    <row r="83" spans="1:14" ht="22.15" customHeight="1">
+    <row r="83" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A83" s="24" t="s">
         <v>113</v>
       </c>
@@ -4905,7 +4902,7 @@
       <c r="M83" s="26"/>
       <c r="N83" s="27"/>
     </row>
-    <row r="84" spans="1:14" ht="22.15" customHeight="1">
+    <row r="84" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A84" s="24" t="s">
         <v>114</v>
       </c>
@@ -4945,7 +4942,7 @@
       <c r="M84" s="26"/>
       <c r="N84" s="27"/>
     </row>
-    <row r="85" spans="1:14" ht="22.15" customHeight="1">
+    <row r="85" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A85" s="24" t="s">
         <v>114</v>
       </c>
@@ -4985,7 +4982,7 @@
       <c r="M85" s="26"/>
       <c r="N85" s="27"/>
     </row>
-    <row r="86" spans="1:14" ht="22.15" customHeight="1">
+    <row r="86" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A86" s="24" t="s">
         <v>114</v>
       </c>
@@ -5025,7 +5022,7 @@
       <c r="M86" s="26"/>
       <c r="N86" s="27"/>
     </row>
-    <row r="87" spans="1:14" ht="22.15" customHeight="1">
+    <row r="87" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A87" s="24" t="s">
         <v>114</v>
       </c>
@@ -5065,7 +5062,7 @@
       <c r="M87" s="26"/>
       <c r="N87" s="27"/>
     </row>
-    <row r="88" spans="1:14" ht="22.15" customHeight="1">
+    <row r="88" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A88" s="24" t="s">
         <v>114</v>
       </c>
@@ -5105,7 +5102,7 @@
       <c r="M88" s="26"/>
       <c r="N88" s="27"/>
     </row>
-    <row r="89" spans="1:14" ht="22.15" customHeight="1">
+    <row r="89" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A89" s="24" t="s">
         <v>90</v>
       </c>
@@ -5130,19 +5127,19 @@
       <c r="H89" s="28">
         <v>15000</v>
       </c>
-      <c r="I89" s="33"/>
-      <c r="J89" s="34"/>
-      <c r="K89" s="34"/>
+      <c r="I89" s="24"/>
+      <c r="J89" s="31"/>
+      <c r="K89" s="31"/>
       <c r="L89" s="25"/>
       <c r="M89" s="26"/>
       <c r="N89" s="27"/>
     </row>
-    <row r="90" spans="1:14" ht="22.15" customHeight="1">
+    <row r="90" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A90" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="B90" s="24" t="s">
-        <v>95</v>
+      <c r="B90" s="30" t="s">
+        <v>115</v>
       </c>
       <c r="C90" s="24" t="s">
         <v>66</v>
@@ -5157,68 +5154,100 @@
         <v>60</v>
       </c>
       <c r="G90" s="28">
-        <v>11943.34</v>
+        <v>23812.5</v>
       </c>
       <c r="H90" s="28">
-        <v>11943.34</v>
-      </c>
-      <c r="I90" s="33"/>
-      <c r="J90" s="34"/>
-      <c r="K90" s="34"/>
+        <v>15000</v>
+      </c>
+      <c r="I90" s="24"/>
+      <c r="J90" s="31"/>
+      <c r="K90" s="31"/>
       <c r="L90" s="25"/>
       <c r="M90" s="26"/>
       <c r="N90" s="27"/>
     </row>
-    <row r="91" spans="1:14" ht="26.1" customHeight="1">
-      <c r="A91" s="18" t="s">
+    <row r="91" spans="1:14" ht="22.15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A91" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B91" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C91" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="D91" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E91" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="F91" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G91" s="28">
+        <v>11943.34</v>
+      </c>
+      <c r="H91" s="28">
+        <v>11943.34</v>
+      </c>
+      <c r="I91" s="24"/>
+      <c r="J91" s="31"/>
+      <c r="K91" s="31"/>
+      <c r="L91" s="25"/>
+      <c r="M91" s="26"/>
+      <c r="N91" s="27"/>
+    </row>
+    <row r="92" spans="1:14" ht="26.1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A92" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="B91" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="C91" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="D91" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="E91" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="F91" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="G91" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="H91" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="I91" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="J91" s="19">
+      <c r="B92" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="C92" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="D92" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="E92" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="F92" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="G92" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="H92" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="I92" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="J92" s="19">
         <f>SUM(J5:J54)</f>
         <v>1872608.537</v>
       </c>
-      <c r="K91" s="19">
+      <c r="K92" s="19">
         <f>SUM(K5:K54)</f>
         <v>1799825.0230000003</v>
       </c>
-      <c r="L91" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="M91" s="19">
+      <c r="L92" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="M92" s="19">
         <f>SUM(M5:M54)</f>
         <v>72783.513999999996</v>
       </c>
-      <c r="N91" s="20">
+      <c r="N92" s="20">
         <f>IF(SUM(K5:K54)&gt;0,SUM(M5:M54)/SUM(K5:K54),0)</f>
         <v>4.0439216629337853E-2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N91" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <autoFilter ref="A1:N92" xr:uid="{00000000-0001-0000-0100-000000000000}">
     <filterColumn colId="0" showButton="0"/>
     <filterColumn colId="1" showButton="0"/>
     <filterColumn colId="2" showButton="0"/>
@@ -5238,16 +5267,16 @@
     <mergeCell ref="A2:N2"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: EPF | Unit Trust | Fixed Deposit | Stocks | Bonds" sqref="C5:C90" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: EPF | Unit Trust | Fixed Deposit | Stocks | Bonds" sqref="C5:C91" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"EPF,Unit Trust,Fixed Deposit,Stocks,Bonds"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Active | Matured | Redeemed | Pending" sqref="E5:E90" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: Active | Matured | Redeemed | Pending" sqref="E5:E91" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"Active,Matured,Redeemed,Pending"</formula1>
     </dataValidation>
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: MYR | USD | SGD | GBP | EUR | AUD | HKD | JPY | CNY" sqref="F5:F90" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Invalid option" error="Please choose: MYR | USD | SGD | GBP | EUR | AUD | HKD | JPY | CNY" sqref="F5:F91" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>"MYR,USD,SGD,GBP,EUR,AUD,HKD,JPY,CNY"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="L5:L90" xr:uid="{00000000-0002-0000-0100-000003000000}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" promptTitle="Date format" prompt="Enter date as YYYY-MM-DD  e.g. 2026-05-19" sqref="L5:L91" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>TRUE</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>